<commit_message>
Add batch cleanup for WeCom and WhatsApp paste
</commit_message>
<xml_diff>
--- a/Geo_TTh_Student_Script_fixed_rows_only.xlsx
+++ b/Geo_TTh_Student_Script_fixed_rows_only.xlsx
@@ -512,7 +512,7 @@
           <t>Calculation</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="15" t="inlineStr">
         <is>
           <t>Additional Comment</t>
         </is>
@@ -4219,7 +4219,7 @@
           <t>Calculation</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="15" t="inlineStr">
         <is>
           <t>Additional Comment</t>
         </is>
@@ -7982,7 +7982,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U200"/>
+  <dimension ref="A1:W200"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63000011444092" defaultRowHeight="15.75"/>
   <cols>
     <col width="18" customWidth="1" style="41" min="1" max="1"/>
@@ -8075,7 +8075,7 @@
           <t>Calculation</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="15" t="inlineStr">
         <is>
           <t>Additional Comment</t>
         </is>
@@ -8108,6 +8108,16 @@
       <c r="U1" s="28" t="inlineStr">
         <is>
           <t>Feedback</t>
+        </is>
+      </c>
+      <c r="V1" s="15" t="inlineStr">
+        <is>
+          <t>Send Error</t>
+        </is>
+      </c>
+      <c r="W1" s="15" t="inlineStr">
+        <is>
+          <t>Last Attempt</t>
         </is>
       </c>
     </row>
@@ -8179,13 +8189,19 @@
       <c r="P2" s="29" t="str"/>
       <c r="Q2" s="29" t="inlineStr">
         <is>
-          <t>Not Generated</t>
+          <t>pasted</t>
         </is>
       </c>
       <c r="R2" s="29" t="n"/>
       <c r="S2" s="29" t="n"/>
       <c r="T2" s="29" t="n"/>
       <c r="U2" s="29" t="n"/>
+      <c r="V2" s="15" t="inlineStr"/>
+      <c r="W2" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-09T00:30:34</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="23" t="inlineStr">
@@ -8403,13 +8419,19 @@
       <c r="P5" s="29" t="str"/>
       <c r="Q5" s="29" t="inlineStr">
         <is>
-          <t>Not Generated</t>
+          <t>pasted</t>
         </is>
       </c>
       <c r="R5" s="29" t="n"/>
       <c r="S5" s="29" t="n"/>
       <c r="T5" s="29" t="n"/>
       <c r="U5" s="29" t="n"/>
+      <c r="V5" s="15" t="inlineStr"/>
+      <c r="W5" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-09T00:20:34</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="23" t="inlineStr">
@@ -8475,13 +8497,23 @@
       <c r="P6" s="29" t="str"/>
       <c r="Q6" s="29" t="inlineStr">
         <is>
-          <t>Not Generated</t>
+          <t>needs_review</t>
         </is>
       </c>
       <c r="R6" s="29" t="n"/>
       <c r="S6" s="29" t="n"/>
       <c r="T6" s="29" t="n"/>
       <c r="U6" s="29" t="n"/>
+      <c r="V6" s="15" t="inlineStr">
+        <is>
+          <t>WhatsApp search key '8204184' did not appear after search input.</t>
+        </is>
+      </c>
+      <c r="W6" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-09T00:26:01</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="23" t="inlineStr">
@@ -8551,13 +8583,19 @@
       <c r="P7" s="29" t="str"/>
       <c r="Q7" s="29" t="inlineStr">
         <is>
-          <t>Not Generated</t>
+          <t>pasted</t>
         </is>
       </c>
       <c r="R7" s="29" t="n"/>
       <c r="S7" s="29" t="n"/>
       <c r="T7" s="29" t="n"/>
       <c r="U7" s="29" t="n"/>
+      <c r="V7" s="15" t="inlineStr"/>
+      <c r="W7" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-09T00:24:53</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="23" t="inlineStr">
@@ -8699,13 +8737,19 @@
       <c r="P9" s="29" t="str"/>
       <c r="Q9" s="29" t="inlineStr">
         <is>
-          <t>Not Generated</t>
+          <t>pasted</t>
         </is>
       </c>
       <c r="R9" s="29" t="n"/>
       <c r="S9" s="29" t="n"/>
       <c r="T9" s="29" t="n"/>
       <c r="U9" s="29" t="n"/>
+      <c r="V9" s="15" t="inlineStr"/>
+      <c r="W9" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-09T00:26:42</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="23" t="inlineStr">
@@ -8927,13 +8971,23 @@
       <c r="P12" s="29" t="str"/>
       <c r="Q12" s="29" t="inlineStr">
         <is>
-          <t>Need Review</t>
+          <t>needs_review</t>
         </is>
       </c>
       <c r="R12" s="29" t="n"/>
       <c r="S12" s="29" t="n"/>
       <c r="T12" s="29" t="n"/>
       <c r="U12" s="29" t="n"/>
+      <c r="V12" s="15" t="inlineStr">
+        <is>
+          <t>WhatsApp chat was not found for search key '8180275'.</t>
+        </is>
+      </c>
+      <c r="W12" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-09T00:34:36</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="23" t="inlineStr">

</xml_diff>

<commit_message>
Improve parent feedback generation
</commit_message>
<xml_diff>
--- a/Geo_TTh_Student_Script_fixed_rows_only.xlsx
+++ b/Geo_TTh_Student_Script_fixed_rows_only.xlsx
@@ -6,6 +6,7 @@
     <sheet name="Geo WF" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="AMC10 Intro" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Geo TTh" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Geo MTWThF" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
 </workbook>
@@ -568,13 +569,41 @@
       <c r="E2" s="19" t="b">
         <v>1</v>
       </c>
-      <c r="F2" s="20" t="n"/>
-      <c r="G2" s="19" t="n"/>
-      <c r="H2" s="19" t="n"/>
-      <c r="I2" s="19" t="n"/>
-      <c r="J2" s="15" t="n"/>
-      <c r="K2" s="15" t="n"/>
-      <c r="L2" s="15" t="n"/>
+      <c r="F2" s="20" t="inlineStr">
+        <is>
+          <t>笔记工整，听课认真，孩子比较安静，但是跟的很好，需要他更多联系3种special angles怎么对应平行，多画图</t>
+        </is>
+      </c>
+      <c r="G2" s="19" t="inlineStr">
+        <is>
+          <t>Chinese</t>
+        </is>
+      </c>
+      <c r="H2" s="19" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="I2" s="19" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J2" s="15" t="inlineStr">
+        <is>
+          <t>Focused</t>
+        </is>
+      </c>
+      <c r="K2" s="15" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="L2" s="15" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
       <c r="M2" s="15" t="n"/>
       <c r="N2" s="15" t="n"/>
       <c r="P2" s="15" t="n"/>
@@ -599,18 +628,46 @@
         <v>7878730</v>
       </c>
       <c r="D3" s="19" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E3" s="19" t="b">
         <v>1</v>
       </c>
-      <c r="F3" s="20" t="n"/>
-      <c r="G3" s="19" t="n"/>
-      <c r="H3" s="19" t="n"/>
-      <c r="I3" s="19" t="n"/>
-      <c r="J3" s="15" t="n"/>
-      <c r="K3" s="15" t="n"/>
-      <c r="L3" s="15" t="n"/>
+      <c r="F3" s="20" t="inlineStr">
+        <is>
+          <t>笔记工整，听课认真，很主动，有问题会主动问我，需要更多练习3种special angles怎么对应平行，多画图。可能还有点不适应集合的做题思路，会有一些小困难，态度很积极，多做练习，相信之后会好起来</t>
+        </is>
+      </c>
+      <c r="G3" s="19" t="inlineStr">
+        <is>
+          <t>Chinese</t>
+        </is>
+      </c>
+      <c r="H3" s="19" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="I3" s="19" t="inlineStr">
+        <is>
+          <t>Excellent</t>
+        </is>
+      </c>
+      <c r="J3" s="15" t="inlineStr">
+        <is>
+          <t>Very Focused</t>
+        </is>
+      </c>
+      <c r="K3" s="15" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="L3" s="15" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
       <c r="M3" s="15" t="n"/>
       <c r="N3" s="15" t="n"/>
       <c r="P3" s="15" t="n"/>
@@ -635,18 +692,46 @@
         <v>7879477</v>
       </c>
       <c r="D4" s="19" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4" s="19" t="b">
         <v>1</v>
       </c>
-      <c r="F4" s="20" t="n"/>
-      <c r="G4" s="19" t="n"/>
-      <c r="H4" s="19" t="n"/>
-      <c r="I4" s="19" t="n"/>
-      <c r="J4" s="15" t="n"/>
-      <c r="K4" s="15" t="n"/>
-      <c r="L4" s="15" t="n"/>
+      <c r="F4" s="20" t="inlineStr">
+        <is>
+          <t>笔记工整，听课认真，因为在AMC10 Intro学过一遍相同的内容，所以掌握的不错，但是对于geometry需要掌握的是如何写好能得分的proof，需要注意AMC10和Geometry的标准不太一样。上课很积极，几乎每个问题他都会举手</t>
+        </is>
+      </c>
+      <c r="G4" s="19" t="inlineStr">
+        <is>
+          <t>Chinese</t>
+        </is>
+      </c>
+      <c r="H4" s="19" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="I4" s="19" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J4" s="15" t="inlineStr">
+        <is>
+          <t>Very Focused</t>
+        </is>
+      </c>
+      <c r="K4" s="15" t="inlineStr">
+        <is>
+          <t>Very Active</t>
+        </is>
+      </c>
+      <c r="L4" s="15" t="inlineStr">
+        <is>
+          <t>Okay</t>
+        </is>
+      </c>
       <c r="M4" s="15" t="n"/>
       <c r="N4" s="15" t="n"/>
       <c r="P4" s="15" t="n"/>
@@ -671,18 +756,46 @@
         <v>7899198</v>
       </c>
       <c r="D5" s="19" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5" s="19" t="b">
-        <v>0</v>
-      </c>
-      <c r="F5" s="20" t="n"/>
-      <c r="G5" s="19" t="n"/>
-      <c r="H5" s="19" t="n"/>
-      <c r="I5" s="19" t="n"/>
-      <c r="J5" s="15" t="n"/>
-      <c r="K5" s="15" t="n"/>
-      <c r="L5" s="15" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="F5" s="20" t="inlineStr">
+        <is>
+          <t>笔记工整，听课认真，很主动，需要更多练习3种special angles怎么对应平行，多画图</t>
+        </is>
+      </c>
+      <c r="G5" s="19" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="H5" s="19" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="I5" s="19" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J5" s="15" t="inlineStr">
+        <is>
+          <t>Focused</t>
+        </is>
+      </c>
+      <c r="K5" s="15" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="L5" s="15" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
       <c r="M5" s="15" t="n"/>
       <c r="N5" s="15" t="n"/>
       <c r="P5" s="15" t="n"/>
@@ -707,18 +820,46 @@
         <v>8397412</v>
       </c>
       <c r="D6" s="19" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E6" s="19" t="b">
         <v>1</v>
       </c>
-      <c r="F6" s="20" t="n"/>
-      <c r="G6" s="19" t="n"/>
-      <c r="H6" s="19" t="n"/>
-      <c r="I6" s="19" t="n"/>
-      <c r="J6" s="15" t="n"/>
-      <c r="K6" s="15" t="n"/>
-      <c r="L6" s="15" t="n"/>
+      <c r="F6" s="20" t="inlineStr">
+        <is>
+          <t>笔记工整，听课认真，总体来说跟的很好，也有跟老师的互动，需要她更多练习3种special angles怎么对应平行，多画图</t>
+        </is>
+      </c>
+      <c r="G6" s="19" t="inlineStr">
+        <is>
+          <t>Chinese</t>
+        </is>
+      </c>
+      <c r="H6" s="19" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="I6" s="19" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J6" s="15" t="inlineStr">
+        <is>
+          <t>Focused</t>
+        </is>
+      </c>
+      <c r="K6" s="15" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="L6" s="15" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
       <c r="M6" s="15" t="n"/>
       <c r="N6" s="15" t="n"/>
       <c r="P6" s="15" t="n"/>
@@ -743,18 +884,46 @@
         <v>8395094</v>
       </c>
       <c r="D7" s="19" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E7" s="19" t="b">
         <v>1</v>
       </c>
-      <c r="F7" s="20" t="n"/>
-      <c r="G7" s="19" t="n"/>
-      <c r="H7" s="19" t="n"/>
-      <c r="I7" s="19" t="n"/>
-      <c r="J7" s="15" t="n"/>
-      <c r="K7" s="15" t="n"/>
-      <c r="L7" s="15" t="n"/>
+      <c r="F7" s="20" t="inlineStr">
+        <is>
+          <t>笔记工整，听课认真，总体来说跟的很好，也有跟老师的互动，需要她更多练习3种special angles怎么对应平行，多画图，有点害羞，孩子有问题可以主动举手问我</t>
+        </is>
+      </c>
+      <c r="G7" s="19" t="inlineStr">
+        <is>
+          <t>Chinese</t>
+        </is>
+      </c>
+      <c r="H7" s="19" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="I7" s="19" t="inlineStr">
+        <is>
+          <t>Excellent</t>
+        </is>
+      </c>
+      <c r="J7" s="15" t="inlineStr">
+        <is>
+          <t>Very Focused</t>
+        </is>
+      </c>
+      <c r="K7" s="15" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="L7" s="15" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
       <c r="M7" s="15" t="n"/>
       <c r="N7" s="15" t="n"/>
       <c r="P7" s="15" t="n"/>
@@ -784,13 +953,41 @@
       <c r="E8" s="19" t="b">
         <v>1</v>
       </c>
-      <c r="F8" s="20" t="n"/>
-      <c r="G8" s="19" t="n"/>
-      <c r="H8" s="19" t="n"/>
-      <c r="I8" s="19" t="n"/>
-      <c r="J8" s="15" t="n"/>
-      <c r="K8" s="15" t="n"/>
-      <c r="L8" s="15" t="n"/>
+      <c r="F8" s="20" t="inlineStr">
+        <is>
+          <t>不怎么记笔记，听课走神很多，需要反复提醒，希望下节课课后有机会可以跟家长谈一谈孩子情况</t>
+        </is>
+      </c>
+      <c r="G8" s="19" t="inlineStr">
+        <is>
+          <t>Chinese</t>
+        </is>
+      </c>
+      <c r="H8" s="19" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="I8" s="19" t="inlineStr">
+        <is>
+          <t>Okay</t>
+        </is>
+      </c>
+      <c r="J8" s="15" t="inlineStr">
+        <is>
+          <t>Sometimes Distracted</t>
+        </is>
+      </c>
+      <c r="K8" s="15" t="inlineStr">
+        <is>
+          <t>Very Active</t>
+        </is>
+      </c>
+      <c r="L8" s="15" t="inlineStr">
+        <is>
+          <t>Okay</t>
+        </is>
+      </c>
       <c r="M8" s="15" t="n"/>
       <c r="N8" s="15" t="n"/>
       <c r="P8" s="15" t="n"/>
@@ -818,15 +1015,43 @@
         <v>0</v>
       </c>
       <c r="E9" s="19" t="b">
-        <v>0</v>
-      </c>
-      <c r="F9" s="20" t="n"/>
-      <c r="G9" s="19" t="n"/>
-      <c r="H9" s="19" t="n"/>
-      <c r="I9" s="19" t="n"/>
-      <c r="J9" s="15" t="n"/>
-      <c r="K9" s="15" t="n"/>
-      <c r="L9" s="15" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="F9" s="20" t="inlineStr">
+        <is>
+          <t>笔记工整，听课认真，跟得很好，互动稍微少一些，但也很积极，很好的理解了材料，第一次自己尝试做证明题就几乎都做对了，写的也很规范</t>
+        </is>
+      </c>
+      <c r="G9" s="19" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="H9" s="19" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="I9" s="19" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J9" s="15" t="inlineStr">
+        <is>
+          <t>Focused</t>
+        </is>
+      </c>
+      <c r="K9" s="15" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="L9" s="15" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
       <c r="M9" s="15" t="n"/>
       <c r="N9" s="15" t="n"/>
       <c r="P9" s="15" t="n"/>
@@ -4276,12 +4501,36 @@
         <v>0</v>
       </c>
       <c r="F2" s="20" t="n"/>
-      <c r="G2" s="20" t="n"/>
-      <c r="H2" s="20" t="n"/>
-      <c r="I2" s="20" t="n"/>
-      <c r="J2" s="20" t="n"/>
-      <c r="K2" s="20" t="n"/>
-      <c r="L2" s="15" t="n"/>
+      <c r="G2" s="20" t="inlineStr">
+        <is>
+          <t>Chinese</t>
+        </is>
+      </c>
+      <c r="H2" s="20" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="I2" s="20" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J2" s="20" t="inlineStr">
+        <is>
+          <t>Focused</t>
+        </is>
+      </c>
+      <c r="K2" s="20" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="L2" s="15" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
       <c r="M2" s="15" t="n"/>
       <c r="N2" s="15" t="n"/>
       <c r="P2" s="15" t="n"/>
@@ -4312,12 +4561,36 @@
         <v>0</v>
       </c>
       <c r="F3" s="20" t="n"/>
-      <c r="G3" s="20" t="n"/>
-      <c r="H3" s="20" t="n"/>
-      <c r="I3" s="20" t="n"/>
-      <c r="J3" s="20" t="n"/>
-      <c r="K3" s="20" t="n"/>
-      <c r="L3" s="15" t="n"/>
+      <c r="G3" s="20" t="inlineStr">
+        <is>
+          <t>Chinese</t>
+        </is>
+      </c>
+      <c r="H3" s="20" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="I3" s="20" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J3" s="20" t="inlineStr">
+        <is>
+          <t>Focused</t>
+        </is>
+      </c>
+      <c r="K3" s="20" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="L3" s="15" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
       <c r="M3" s="15" t="n"/>
       <c r="N3" s="15" t="n"/>
       <c r="P3" s="15" t="n"/>
@@ -4348,12 +4621,36 @@
         <v>0</v>
       </c>
       <c r="F4" s="20" t="n"/>
-      <c r="G4" s="20" t="n"/>
-      <c r="H4" s="20" t="n"/>
-      <c r="I4" s="20" t="n"/>
-      <c r="J4" s="20" t="n"/>
-      <c r="K4" s="20" t="n"/>
-      <c r="L4" s="15" t="n"/>
+      <c r="G4" s="20" t="inlineStr">
+        <is>
+          <t>Chinese</t>
+        </is>
+      </c>
+      <c r="H4" s="20" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="I4" s="20" t="inlineStr">
+        <is>
+          <t>Excellent</t>
+        </is>
+      </c>
+      <c r="J4" s="20" t="inlineStr">
+        <is>
+          <t>Very Focused</t>
+        </is>
+      </c>
+      <c r="K4" s="20" t="inlineStr">
+        <is>
+          <t>Very Active</t>
+        </is>
+      </c>
+      <c r="L4" s="15" t="inlineStr">
+        <is>
+          <t>Okay</t>
+        </is>
+      </c>
       <c r="M4" s="15" t="n"/>
       <c r="N4" s="15" t="n"/>
       <c r="P4" s="15" t="n"/>
@@ -4384,12 +4681,36 @@
         <v>0</v>
       </c>
       <c r="F5" s="20" t="n"/>
-      <c r="G5" s="20" t="n"/>
-      <c r="H5" s="20" t="n"/>
-      <c r="I5" s="20" t="n"/>
-      <c r="J5" s="20" t="n"/>
-      <c r="K5" s="20" t="n"/>
-      <c r="L5" s="15" t="n"/>
+      <c r="G5" s="20" t="inlineStr">
+        <is>
+          <t>Chinese</t>
+        </is>
+      </c>
+      <c r="H5" s="20" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="I5" s="20" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J5" s="20" t="inlineStr">
+        <is>
+          <t>Focused</t>
+        </is>
+      </c>
+      <c r="K5" s="20" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="L5" s="15" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
       <c r="M5" s="15" t="n"/>
       <c r="N5" s="15" t="n"/>
       <c r="P5" s="15" t="n"/>
@@ -4420,12 +4741,36 @@
         <v>0</v>
       </c>
       <c r="F6" s="20" t="n"/>
-      <c r="G6" s="20" t="n"/>
-      <c r="H6" s="20" t="n"/>
-      <c r="I6" s="20" t="n"/>
-      <c r="J6" s="20" t="n"/>
-      <c r="K6" s="20" t="n"/>
-      <c r="L6" s="15" t="n"/>
+      <c r="G6" s="20" t="inlineStr">
+        <is>
+          <t>Chinese</t>
+        </is>
+      </c>
+      <c r="H6" s="20" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="I6" s="20" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J6" s="20" t="inlineStr">
+        <is>
+          <t>Focused</t>
+        </is>
+      </c>
+      <c r="K6" s="20" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="L6" s="15" t="inlineStr">
+        <is>
+          <t>Okay</t>
+        </is>
+      </c>
       <c r="M6" s="15" t="n"/>
       <c r="N6" s="15" t="n"/>
       <c r="P6" s="15" t="n"/>
@@ -4456,12 +4801,36 @@
         <v>0</v>
       </c>
       <c r="F7" s="20" t="n"/>
-      <c r="G7" s="20" t="n"/>
-      <c r="H7" s="20" t="n"/>
-      <c r="I7" s="20" t="n"/>
-      <c r="J7" s="20" t="n"/>
-      <c r="K7" s="20" t="n"/>
-      <c r="L7" s="15" t="n"/>
+      <c r="G7" s="20" t="inlineStr">
+        <is>
+          <t>Chinese</t>
+        </is>
+      </c>
+      <c r="H7" s="20" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="I7" s="20" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J7" s="20" t="inlineStr">
+        <is>
+          <t>Focused</t>
+        </is>
+      </c>
+      <c r="K7" s="20" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="L7" s="15" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
       <c r="M7" s="15" t="n"/>
       <c r="N7" s="15" t="n"/>
       <c r="P7" s="15" t="n"/>
@@ -4492,12 +4861,36 @@
         <v>0</v>
       </c>
       <c r="F8" s="20" t="n"/>
-      <c r="G8" s="20" t="n"/>
-      <c r="H8" s="20" t="n"/>
-      <c r="I8" s="20" t="n"/>
-      <c r="J8" s="20" t="n"/>
-      <c r="K8" s="20" t="n"/>
-      <c r="L8" s="15" t="n"/>
+      <c r="G8" s="20" t="inlineStr">
+        <is>
+          <t>Chinese</t>
+        </is>
+      </c>
+      <c r="H8" s="20" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="I8" s="20" t="inlineStr">
+        <is>
+          <t>Excellent</t>
+        </is>
+      </c>
+      <c r="J8" s="20" t="inlineStr">
+        <is>
+          <t>Very Focused</t>
+        </is>
+      </c>
+      <c r="K8" s="20" t="inlineStr">
+        <is>
+          <t>Very Active</t>
+        </is>
+      </c>
+      <c r="L8" s="15" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
       <c r="M8" s="15" t="n"/>
       <c r="N8" s="15" t="n"/>
       <c r="P8" s="15" t="n"/>
@@ -4528,12 +4921,36 @@
         <v>0</v>
       </c>
       <c r="F9" s="20" t="n"/>
-      <c r="G9" s="20" t="n"/>
-      <c r="H9" s="20" t="n"/>
-      <c r="I9" s="20" t="n"/>
-      <c r="J9" s="20" t="n"/>
-      <c r="K9" s="20" t="n"/>
-      <c r="L9" s="15" t="n"/>
+      <c r="G9" s="20" t="inlineStr">
+        <is>
+          <t>Chinese</t>
+        </is>
+      </c>
+      <c r="H9" s="20" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="I9" s="20" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J9" s="20" t="inlineStr">
+        <is>
+          <t>Focused</t>
+        </is>
+      </c>
+      <c r="K9" s="20" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="L9" s="15" t="inlineStr">
+        <is>
+          <t>Okay</t>
+        </is>
+      </c>
       <c r="M9" s="15" t="n"/>
       <c r="N9" s="15" t="n"/>
       <c r="P9" s="15" t="n"/>
@@ -4564,12 +4981,36 @@
         <v>0</v>
       </c>
       <c r="F10" s="20" t="n"/>
-      <c r="G10" s="20" t="n"/>
-      <c r="H10" s="20" t="n"/>
-      <c r="I10" s="20" t="n"/>
-      <c r="J10" s="20" t="n"/>
-      <c r="K10" s="20" t="n"/>
-      <c r="L10" s="15" t="n"/>
+      <c r="G10" s="20" t="inlineStr">
+        <is>
+          <t>Chinese</t>
+        </is>
+      </c>
+      <c r="H10" s="20" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="I10" s="20" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J10" s="20" t="inlineStr">
+        <is>
+          <t>Focused</t>
+        </is>
+      </c>
+      <c r="K10" s="20" t="inlineStr">
+        <is>
+          <t>Very Active</t>
+        </is>
+      </c>
+      <c r="L10" s="15" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
       <c r="M10" s="15" t="n"/>
       <c r="N10" s="15" t="n"/>
       <c r="P10" s="15" t="n"/>
@@ -4600,12 +5041,36 @@
         <v>0</v>
       </c>
       <c r="F11" s="20" t="n"/>
-      <c r="G11" s="20" t="n"/>
-      <c r="H11" s="20" t="n"/>
-      <c r="I11" s="20" t="n"/>
-      <c r="J11" s="20" t="n"/>
-      <c r="K11" s="20" t="n"/>
-      <c r="L11" s="15" t="n"/>
+      <c r="G11" s="20" t="inlineStr">
+        <is>
+          <t>Chinese</t>
+        </is>
+      </c>
+      <c r="H11" s="20" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="I11" s="20" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J11" s="20" t="inlineStr">
+        <is>
+          <t>Focused</t>
+        </is>
+      </c>
+      <c r="K11" s="20" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="L11" s="15" t="inlineStr">
+        <is>
+          <t>Okay</t>
+        </is>
+      </c>
       <c r="M11" s="15" t="n"/>
       <c r="N11" s="15" t="n"/>
       <c r="P11" s="15" t="n"/>
@@ -4636,12 +5101,36 @@
         <v>0</v>
       </c>
       <c r="F12" s="20" t="n"/>
-      <c r="G12" s="20" t="n"/>
-      <c r="H12" s="20" t="n"/>
-      <c r="I12" s="20" t="n"/>
-      <c r="J12" s="20" t="n"/>
-      <c r="K12" s="20" t="n"/>
-      <c r="L12" s="15" t="n"/>
+      <c r="G12" s="20" t="inlineStr">
+        <is>
+          <t>Chinese</t>
+        </is>
+      </c>
+      <c r="H12" s="20" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="I12" s="20" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J12" s="20" t="inlineStr">
+        <is>
+          <t>Focused</t>
+        </is>
+      </c>
+      <c r="K12" s="20" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="L12" s="15" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
       <c r="M12" s="15" t="n"/>
       <c r="N12" s="15" t="n"/>
       <c r="P12" s="15" t="n"/>
@@ -4672,12 +5161,36 @@
         <v>0</v>
       </c>
       <c r="F13" s="20" t="n"/>
-      <c r="G13" s="20" t="n"/>
-      <c r="H13" s="20" t="n"/>
-      <c r="I13" s="20" t="n"/>
-      <c r="J13" s="20" t="n"/>
-      <c r="K13" s="20" t="n"/>
-      <c r="L13" s="15" t="n"/>
+      <c r="G13" s="20" t="inlineStr">
+        <is>
+          <t>Chinese</t>
+        </is>
+      </c>
+      <c r="H13" s="20" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="I13" s="20" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J13" s="20" t="inlineStr">
+        <is>
+          <t>Focused</t>
+        </is>
+      </c>
+      <c r="K13" s="20" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="L13" s="15" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
       <c r="M13" s="15" t="n"/>
       <c r="N13" s="15" t="n"/>
       <c r="P13" s="15" t="n"/>
@@ -4708,12 +5221,36 @@
         <v>0</v>
       </c>
       <c r="F14" s="20" t="n"/>
-      <c r="G14" s="20" t="n"/>
-      <c r="H14" s="20" t="n"/>
-      <c r="I14" s="20" t="n"/>
-      <c r="J14" s="20" t="n"/>
-      <c r="K14" s="20" t="n"/>
-      <c r="L14" s="15" t="n"/>
+      <c r="G14" s="20" t="inlineStr">
+        <is>
+          <t>Chinese</t>
+        </is>
+      </c>
+      <c r="H14" s="20" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="I14" s="20" t="inlineStr">
+        <is>
+          <t>Excellent</t>
+        </is>
+      </c>
+      <c r="J14" s="20" t="inlineStr">
+        <is>
+          <t>Focused</t>
+        </is>
+      </c>
+      <c r="K14" s="20" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="L14" s="15" t="inlineStr">
+        <is>
+          <t>Okay</t>
+        </is>
+      </c>
       <c r="M14" s="15" t="n"/>
       <c r="N14" s="15" t="n"/>
       <c r="P14" s="15" t="n"/>
@@ -4744,12 +5281,36 @@
         <v>0</v>
       </c>
       <c r="F15" s="20" t="n"/>
-      <c r="G15" s="20" t="n"/>
-      <c r="H15" s="20" t="n"/>
-      <c r="I15" s="20" t="n"/>
-      <c r="J15" s="20" t="n"/>
-      <c r="K15" s="20" t="n"/>
-      <c r="L15" s="15" t="n"/>
+      <c r="G15" s="20" t="inlineStr">
+        <is>
+          <t>Chinese</t>
+        </is>
+      </c>
+      <c r="H15" s="20" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="I15" s="20" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J15" s="20" t="inlineStr">
+        <is>
+          <t>Focused</t>
+        </is>
+      </c>
+      <c r="K15" s="20" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="L15" s="15" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
       <c r="M15" s="15" t="n"/>
       <c r="N15" s="15" t="n"/>
       <c r="P15" s="15" t="n"/>
@@ -4780,12 +5341,36 @@
         <v>0</v>
       </c>
       <c r="F16" s="20" t="n"/>
-      <c r="G16" s="20" t="n"/>
-      <c r="H16" s="20" t="n"/>
-      <c r="I16" s="20" t="n"/>
-      <c r="J16" s="20" t="n"/>
-      <c r="K16" s="20" t="n"/>
-      <c r="L16" s="15" t="n"/>
+      <c r="G16" s="20" t="inlineStr">
+        <is>
+          <t>Chinese</t>
+        </is>
+      </c>
+      <c r="H16" s="20" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="I16" s="20" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J16" s="20" t="inlineStr">
+        <is>
+          <t>Focused</t>
+        </is>
+      </c>
+      <c r="K16" s="20" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="L16" s="15" t="inlineStr">
+        <is>
+          <t>Okay</t>
+        </is>
+      </c>
       <c r="M16" s="15" t="n"/>
       <c r="N16" s="15" t="n"/>
       <c r="P16" s="15" t="n"/>
@@ -4796,25 +5381,11 @@
       <c r="U16" s="15" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="20" t="inlineStr">
-        <is>
-          <t>Alisha</t>
-        </is>
-      </c>
-      <c r="B17" s="20" t="inlineStr">
-        <is>
-          <t>Sutar</t>
-        </is>
-      </c>
-      <c r="C17" s="20" t="n">
-        <v>8256341</v>
-      </c>
-      <c r="D17" s="20" t="b">
-        <v>0</v>
-      </c>
-      <c r="E17" s="20" t="b">
-        <v>0</v>
-      </c>
+      <c r="A17" s="20" t="n"/>
+      <c r="B17" s="20" t="n"/>
+      <c r="C17" s="20" t="n"/>
+      <c r="D17" s="20" t="n"/>
+      <c r="E17" s="20" t="n"/>
       <c r="F17" s="20" t="n"/>
       <c r="G17" s="20" t="n"/>
       <c r="H17" s="20" t="n"/>
@@ -8001,7 +8572,13 @@
     <col width="18" customWidth="1" style="41" min="14" max="14"/>
     <col width="24" customWidth="1" style="41" min="15" max="15"/>
     <col width="18" customWidth="1" style="41" min="16" max="16"/>
+    <col width="13" customWidth="1" style="41" min="17" max="17"/>
+    <col width="13" customWidth="1" style="41" min="18" max="18"/>
+    <col width="13" customWidth="1" style="41" min="19" max="19"/>
     <col width="38" customWidth="1" style="41" min="20" max="20"/>
+    <col width="13" customWidth="1" style="41" min="21" max="21"/>
+    <col width="13" customWidth="1" style="41" min="22" max="22"/>
+    <col width="13" customWidth="1" style="41" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8176,27 +8753,15 @@
           <t>Fast but Needs Care</t>
         </is>
       </c>
-      <c r="M2" s="23" t="inlineStr">
-        <is>
-          <t>Not Observed</t>
-        </is>
-      </c>
-      <c r="N2" s="23" t="inlineStr">
-        <is>
-          <t>Not Observed</t>
-        </is>
-      </c>
-      <c r="P2" s="29" t="str"/>
-      <c r="Q2" s="29" t="inlineStr">
-        <is>
-          <t>pasted</t>
-        </is>
-      </c>
+      <c r="M2" s="23" t="n"/>
+      <c r="N2" s="23" t="n"/>
+      <c r="P2" s="29" t="n"/>
+      <c r="Q2" s="29" t="n"/>
       <c r="R2" s="29" t="n"/>
       <c r="S2" s="29" t="n"/>
       <c r="T2" s="29" t="n"/>
       <c r="U2" s="29" t="n"/>
-      <c r="V2" s="15" t="inlineStr"/>
+      <c r="V2" s="15" t="n"/>
       <c r="W2" s="15" t="inlineStr">
         <is>
           <t>2026-06-09T00:30:34</t>
@@ -8258,22 +8823,10 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="M3" s="23" t="inlineStr">
-        <is>
-          <t>Not Observed</t>
-        </is>
-      </c>
-      <c r="N3" s="23" t="inlineStr">
-        <is>
-          <t>Not Observed</t>
-        </is>
-      </c>
-      <c r="P3" s="29" t="str"/>
-      <c r="Q3" s="29" t="inlineStr">
-        <is>
-          <t>Not Generated</t>
-        </is>
-      </c>
+      <c r="M3" s="23" t="n"/>
+      <c r="N3" s="23" t="n"/>
+      <c r="P3" s="29" t="n"/>
+      <c r="Q3" s="29" t="n"/>
       <c r="R3" s="29" t="n"/>
       <c r="S3" s="29" t="n"/>
       <c r="T3" s="29" t="n"/>
@@ -8334,22 +8887,10 @@
           <t>Good</t>
         </is>
       </c>
-      <c r="M4" s="23" t="inlineStr">
-        <is>
-          <t>Needs Practice</t>
-        </is>
-      </c>
-      <c r="N4" s="23" t="inlineStr">
-        <is>
-          <t>Not Observed</t>
-        </is>
-      </c>
-      <c r="P4" s="29" t="str"/>
-      <c r="Q4" s="29" t="inlineStr">
-        <is>
-          <t>Not Generated</t>
-        </is>
-      </c>
+      <c r="M4" s="23" t="n"/>
+      <c r="N4" s="23" t="n"/>
+      <c r="P4" s="29" t="n"/>
+      <c r="Q4" s="29" t="n"/>
       <c r="R4" s="29" t="n"/>
       <c r="S4" s="29" t="n"/>
       <c r="T4" s="29" t="n"/>
@@ -8406,27 +8947,15 @@
           <t>Not Observed</t>
         </is>
       </c>
-      <c r="M5" s="23" t="inlineStr">
-        <is>
-          <t>Not Observed</t>
-        </is>
-      </c>
-      <c r="N5" s="23" t="inlineStr">
-        <is>
-          <t>Not Observed</t>
-        </is>
-      </c>
-      <c r="P5" s="29" t="str"/>
-      <c r="Q5" s="29" t="inlineStr">
-        <is>
-          <t>pasted</t>
-        </is>
-      </c>
+      <c r="M5" s="23" t="n"/>
+      <c r="N5" s="23" t="n"/>
+      <c r="P5" s="29" t="n"/>
+      <c r="Q5" s="29" t="n"/>
       <c r="R5" s="29" t="n"/>
       <c r="S5" s="29" t="n"/>
       <c r="T5" s="29" t="n"/>
       <c r="U5" s="29" t="n"/>
-      <c r="V5" s="15" t="inlineStr"/>
+      <c r="V5" s="15" t="n"/>
       <c r="W5" s="15" t="inlineStr">
         <is>
           <t>2026-06-09T00:20:34</t>
@@ -8484,22 +9013,10 @@
           <t>Not Observed</t>
         </is>
       </c>
-      <c r="M6" s="23" t="inlineStr">
-        <is>
-          <t>Not Observed</t>
-        </is>
-      </c>
-      <c r="N6" s="23" t="inlineStr">
-        <is>
-          <t>Not Observed</t>
-        </is>
-      </c>
-      <c r="P6" s="29" t="str"/>
-      <c r="Q6" s="29" t="inlineStr">
-        <is>
-          <t>needs_review</t>
-        </is>
-      </c>
+      <c r="M6" s="23" t="n"/>
+      <c r="N6" s="23" t="n"/>
+      <c r="P6" s="29" t="n"/>
+      <c r="Q6" s="29" t="n"/>
       <c r="R6" s="29" t="n"/>
       <c r="S6" s="29" t="n"/>
       <c r="T6" s="29" t="n"/>
@@ -8570,27 +9087,15 @@
           <t>Good</t>
         </is>
       </c>
-      <c r="M7" s="23" t="inlineStr">
-        <is>
-          <t>Needs Practice</t>
-        </is>
-      </c>
-      <c r="N7" s="23" t="inlineStr">
-        <is>
-          <t>Not Observed</t>
-        </is>
-      </c>
-      <c r="P7" s="29" t="str"/>
-      <c r="Q7" s="29" t="inlineStr">
-        <is>
-          <t>pasted</t>
-        </is>
-      </c>
+      <c r="M7" s="23" t="n"/>
+      <c r="N7" s="23" t="n"/>
+      <c r="P7" s="29" t="n"/>
+      <c r="Q7" s="29" t="n"/>
       <c r="R7" s="29" t="n"/>
       <c r="S7" s="29" t="n"/>
       <c r="T7" s="29" t="n"/>
       <c r="U7" s="29" t="n"/>
-      <c r="V7" s="15" t="inlineStr"/>
+      <c r="V7" s="15" t="n"/>
       <c r="W7" s="15" t="inlineStr">
         <is>
           <t>2026-06-09T00:24:53</t>
@@ -8612,14 +9117,14 @@
         <v>7886071</v>
       </c>
       <c r="D8" s="23" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E8" s="23" t="b">
         <v>1</v>
       </c>
       <c r="F8" s="23" t="inlineStr">
         <is>
-          <t>笔记公正，听课认真，学有余力，会帮助旁边不会的小朋友</t>
+          <t>笔记工整，听课认真，学有余力，会帮助旁边不会的小朋友</t>
         </is>
       </c>
       <c r="G8" s="23" t="inlineStr">
@@ -8634,40 +9139,28 @@
       </c>
       <c r="I8" s="23" t="inlineStr">
         <is>
+          <t>Focused</t>
+        </is>
+      </c>
+      <c r="J8" s="23" t="inlineStr">
+        <is>
+          <t>Sometimes Distracted</t>
+        </is>
+      </c>
+      <c r="K8" s="23" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="L8" s="23" t="inlineStr">
+        <is>
           <t>Good</t>
         </is>
       </c>
-      <c r="J8" s="23" t="inlineStr">
-        <is>
-          <t>Focused</t>
-        </is>
-      </c>
-      <c r="K8" s="23" t="inlineStr">
-        <is>
-          <t>Helpful</t>
-        </is>
-      </c>
-      <c r="L8" s="23" t="inlineStr">
-        <is>
-          <t>Excellent</t>
-        </is>
-      </c>
-      <c r="M8" s="23" t="inlineStr">
-        <is>
-          <t>Strong</t>
-        </is>
-      </c>
-      <c r="N8" s="23" t="inlineStr">
-        <is>
-          <t>Good</t>
-        </is>
-      </c>
-      <c r="P8" s="29" t="str"/>
-      <c r="Q8" s="29" t="inlineStr">
-        <is>
-          <t>Not Generated</t>
-        </is>
-      </c>
+      <c r="M8" s="23" t="n"/>
+      <c r="N8" s="23" t="n"/>
+      <c r="P8" s="29" t="n"/>
+      <c r="Q8" s="29" t="n"/>
       <c r="R8" s="29" t="n"/>
       <c r="S8" s="29" t="n"/>
       <c r="T8" s="29" t="n"/>
@@ -8693,7 +9186,11 @@
       <c r="E9" s="23" t="b">
         <v>1</v>
       </c>
-      <c r="F9" s="23" t="n"/>
+      <c r="F9" s="23" t="inlineStr">
+        <is>
+          <t>笔记工整，听课认真，会和Nanette一起讨论问题</t>
+        </is>
+      </c>
       <c r="G9" s="23" t="inlineStr">
         <is>
           <t>Chinese</t>
@@ -8706,45 +9203,33 @@
       </c>
       <c r="I9" s="23" t="inlineStr">
         <is>
-          <t>Not Observed</t>
+          <t>Focused</t>
         </is>
       </c>
       <c r="J9" s="23" t="inlineStr">
         <is>
-          <t>Not Observed</t>
+          <t>Sometimes Distracted</t>
         </is>
       </c>
       <c r="K9" s="23" t="inlineStr">
         <is>
-          <t>Not Observed</t>
+          <t>Average</t>
         </is>
       </c>
       <c r="L9" s="23" t="inlineStr">
         <is>
-          <t>Not Observed</t>
-        </is>
-      </c>
-      <c r="M9" s="23" t="inlineStr">
-        <is>
-          <t>Not Observed</t>
-        </is>
-      </c>
-      <c r="N9" s="23" t="inlineStr">
-        <is>
-          <t>Not Observed</t>
-        </is>
-      </c>
-      <c r="P9" s="29" t="str"/>
-      <c r="Q9" s="29" t="inlineStr">
-        <is>
-          <t>pasted</t>
-        </is>
-      </c>
+          <t>Okay</t>
+        </is>
+      </c>
+      <c r="M9" s="23" t="n"/>
+      <c r="N9" s="23" t="n"/>
+      <c r="P9" s="29" t="n"/>
+      <c r="Q9" s="29" t="n"/>
       <c r="R9" s="29" t="n"/>
       <c r="S9" s="29" t="n"/>
       <c r="T9" s="29" t="n"/>
       <c r="U9" s="29" t="n"/>
-      <c r="V9" s="15" t="inlineStr"/>
+      <c r="V9" s="15" t="n"/>
       <c r="W9" s="15" t="inlineStr">
         <is>
           <t>2026-06-09T00:26:42</t>
@@ -8806,22 +9291,10 @@
           <t>Needs Support</t>
         </is>
       </c>
-      <c r="M10" s="23" t="inlineStr">
-        <is>
-          <t>Good with Hint</t>
-        </is>
-      </c>
-      <c r="N10" s="23" t="inlineStr">
-        <is>
-          <t>Not Observed</t>
-        </is>
-      </c>
-      <c r="P10" s="29" t="str"/>
-      <c r="Q10" s="29" t="inlineStr">
-        <is>
-          <t>Not Generated</t>
-        </is>
-      </c>
+      <c r="M10" s="23" t="n"/>
+      <c r="N10" s="23" t="n"/>
+      <c r="P10" s="29" t="n"/>
+      <c r="Q10" s="29" t="n"/>
       <c r="R10" s="29" t="n"/>
       <c r="S10" s="29" t="n"/>
       <c r="T10" s="29" t="n"/>
@@ -8882,22 +9355,10 @@
           <t>Slow but Thoughtful</t>
         </is>
       </c>
-      <c r="M11" s="23" t="inlineStr">
-        <is>
-          <t>Not Observed</t>
-        </is>
-      </c>
-      <c r="N11" s="23" t="inlineStr">
-        <is>
-          <t>Not Observed</t>
-        </is>
-      </c>
-      <c r="P11" s="29" t="str"/>
-      <c r="Q11" s="29" t="inlineStr">
-        <is>
-          <t>Not Generated</t>
-        </is>
-      </c>
+      <c r="M11" s="23" t="n"/>
+      <c r="N11" s="23" t="n"/>
+      <c r="P11" s="29" t="n"/>
+      <c r="Q11" s="29" t="n"/>
       <c r="R11" s="29" t="n"/>
       <c r="S11" s="29" t="n"/>
       <c r="T11" s="29" t="n"/>
@@ -8958,22 +9419,10 @@
           <t>Good but Rushed</t>
         </is>
       </c>
-      <c r="M12" s="23" t="inlineStr">
-        <is>
-          <t>Strong</t>
-        </is>
-      </c>
-      <c r="N12" s="23" t="inlineStr">
-        <is>
-          <t>Needs More Care</t>
-        </is>
-      </c>
-      <c r="P12" s="29" t="str"/>
-      <c r="Q12" s="29" t="inlineStr">
-        <is>
-          <t>needs_review</t>
-        </is>
-      </c>
+      <c r="M12" s="23" t="n"/>
+      <c r="N12" s="23" t="n"/>
+      <c r="P12" s="29" t="n"/>
+      <c r="Q12" s="29" t="n"/>
       <c r="R12" s="29" t="n"/>
       <c r="S12" s="29" t="n"/>
       <c r="T12" s="29" t="n"/>
@@ -9044,22 +9493,10 @@
           <t>Good</t>
         </is>
       </c>
-      <c r="M13" s="23" t="inlineStr">
-        <is>
-          <t>Not Observed</t>
-        </is>
-      </c>
-      <c r="N13" s="23" t="inlineStr">
-        <is>
-          <t>Not Observed</t>
-        </is>
-      </c>
-      <c r="P13" s="29" t="str"/>
-      <c r="Q13" s="29" t="inlineStr">
-        <is>
-          <t>Need Review</t>
-        </is>
-      </c>
+      <c r="M13" s="23" t="n"/>
+      <c r="N13" s="23" t="n"/>
+      <c r="P13" s="29" t="n"/>
+      <c r="Q13" s="29" t="n"/>
       <c r="R13" s="29" t="n"/>
       <c r="S13" s="29" t="n"/>
       <c r="T13" s="29" t="n"/>
@@ -9097,7 +9534,7 @@
       </c>
       <c r="H14" s="23" t="inlineStr">
         <is>
-          <t>Absent</t>
+          <t>Present</t>
         </is>
       </c>
       <c r="I14" s="23" t="inlineStr">
@@ -9120,22 +9557,10 @@
           <t>Not Observed</t>
         </is>
       </c>
-      <c r="M14" s="23" t="inlineStr">
-        <is>
-          <t>Not Observed</t>
-        </is>
-      </c>
-      <c r="N14" s="23" t="inlineStr">
-        <is>
-          <t>Not Observed</t>
-        </is>
-      </c>
-      <c r="P14" s="29" t="str"/>
-      <c r="Q14" s="29" t="inlineStr">
-        <is>
-          <t>Need Review</t>
-        </is>
-      </c>
+      <c r="M14" s="23" t="n"/>
+      <c r="N14" s="23" t="n"/>
+      <c r="P14" s="29" t="n"/>
+      <c r="Q14" s="29" t="n"/>
       <c r="R14" s="29" t="n"/>
       <c r="S14" s="29" t="n"/>
       <c r="T14" s="29" t="n"/>
@@ -9196,22 +9621,10 @@
           <t>Good</t>
         </is>
       </c>
-      <c r="M15" s="23" t="inlineStr">
-        <is>
-          <t>Not Observed</t>
-        </is>
-      </c>
-      <c r="N15" s="23" t="inlineStr">
-        <is>
-          <t>Needs More Care</t>
-        </is>
-      </c>
-      <c r="P15" s="29" t="str"/>
-      <c r="Q15" s="29" t="inlineStr">
-        <is>
-          <t>Not Generated</t>
-        </is>
-      </c>
+      <c r="M15" s="23" t="n"/>
+      <c r="N15" s="23" t="n"/>
+      <c r="P15" s="29" t="n"/>
+      <c r="Q15" s="29" t="n"/>
       <c r="R15" s="29" t="n"/>
       <c r="S15" s="29" t="n"/>
       <c r="T15" s="29" t="n"/>
@@ -9237,7 +9650,11 @@
       <c r="E16" s="23" t="b">
         <v>1</v>
       </c>
-      <c r="F16" s="23" t="n"/>
+      <c r="F16" s="23" t="inlineStr">
+        <is>
+          <t>笔记工整，听课认真，同学总的来说动作很快，但是有的时候会在讲题的时候写，如果可以让他先听一遍在记录下来应该能更好的掌握内容</t>
+        </is>
+      </c>
       <c r="G16" s="23" t="inlineStr">
         <is>
           <t>Chinese</t>
@@ -9245,7 +9662,7 @@
       </c>
       <c r="H16" s="23" t="inlineStr">
         <is>
-          <t>Absent</t>
+          <t>Present</t>
         </is>
       </c>
       <c r="I16" s="23" t="inlineStr">
@@ -9268,22 +9685,10 @@
           <t>Not Observed</t>
         </is>
       </c>
-      <c r="M16" s="23" t="inlineStr">
-        <is>
-          <t>Not Observed</t>
-        </is>
-      </c>
-      <c r="N16" s="23" t="inlineStr">
-        <is>
-          <t>Not Observed</t>
-        </is>
-      </c>
-      <c r="P16" s="29" t="str"/>
-      <c r="Q16" s="29" t="inlineStr">
-        <is>
-          <t>Need Review</t>
-        </is>
-      </c>
+      <c r="M16" s="23" t="n"/>
+      <c r="N16" s="23" t="n"/>
+      <c r="P16" s="29" t="n"/>
+      <c r="Q16" s="29" t="n"/>
       <c r="R16" s="29" t="n"/>
       <c r="S16" s="29" t="n"/>
       <c r="T16" s="29" t="n"/>
@@ -9304,7 +9709,7 @@
         <v>8193635</v>
       </c>
       <c r="D17" s="23" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E17" s="23" t="b">
         <v>1</v>
@@ -9344,22 +9749,10 @@
           <t>Needs Support</t>
         </is>
       </c>
-      <c r="M17" s="23" t="inlineStr">
-        <is>
-          <t>Not Observed</t>
-        </is>
-      </c>
-      <c r="N17" s="23" t="inlineStr">
-        <is>
-          <t>Not Observed</t>
-        </is>
-      </c>
-      <c r="P17" s="29" t="str"/>
-      <c r="Q17" s="29" t="inlineStr">
-        <is>
-          <t>Need Review</t>
-        </is>
-      </c>
+      <c r="M17" s="23" t="n"/>
+      <c r="N17" s="23" t="n"/>
+      <c r="P17" s="29" t="n"/>
+      <c r="Q17" s="29" t="n"/>
       <c r="R17" s="29" t="n"/>
       <c r="S17" s="29" t="n"/>
       <c r="T17" s="29" t="n"/>
@@ -9416,22 +9809,10 @@
           <t>Not Observed</t>
         </is>
       </c>
-      <c r="M18" s="23" t="inlineStr">
-        <is>
-          <t>Not Observed</t>
-        </is>
-      </c>
-      <c r="N18" s="23" t="inlineStr">
-        <is>
-          <t>Not Observed</t>
-        </is>
-      </c>
-      <c r="P18" s="29" t="str"/>
-      <c r="Q18" s="29" t="inlineStr">
-        <is>
-          <t>Not Generated</t>
-        </is>
-      </c>
+      <c r="M18" s="23" t="n"/>
+      <c r="N18" s="23" t="n"/>
+      <c r="P18" s="29" t="n"/>
+      <c r="Q18" s="29" t="n"/>
       <c r="R18" s="29" t="n"/>
       <c r="S18" s="29" t="n"/>
       <c r="T18" s="29" t="n"/>
@@ -9492,22 +9873,10 @@
           <t>High Accuracy</t>
         </is>
       </c>
-      <c r="M19" s="23" t="inlineStr">
-        <is>
-          <t>Strong</t>
-        </is>
-      </c>
-      <c r="N19" s="23" t="inlineStr">
-        <is>
-          <t>Good</t>
-        </is>
-      </c>
-      <c r="P19" s="29" t="str"/>
-      <c r="Q19" s="29" t="inlineStr">
-        <is>
-          <t>Not Generated</t>
-        </is>
-      </c>
+      <c r="M19" s="23" t="n"/>
+      <c r="N19" s="23" t="n"/>
+      <c r="P19" s="29" t="n"/>
+      <c r="Q19" s="29" t="n"/>
       <c r="R19" s="29" t="n"/>
       <c r="S19" s="29" t="n"/>
       <c r="T19" s="29" t="n"/>
@@ -9528,7 +9897,7 @@
         <v>8397642</v>
       </c>
       <c r="D20" s="23" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E20" s="23" t="b">
         <v>1</v>
@@ -9568,22 +9937,10 @@
           <t>Good</t>
         </is>
       </c>
-      <c r="M20" s="23" t="inlineStr">
-        <is>
-          <t>Not Observed</t>
-        </is>
-      </c>
-      <c r="N20" s="23" t="inlineStr">
-        <is>
-          <t>Not Observed</t>
-        </is>
-      </c>
-      <c r="P20" s="29" t="str"/>
-      <c r="Q20" s="29" t="inlineStr">
-        <is>
-          <t>Not Generated</t>
-        </is>
-      </c>
+      <c r="M20" s="23" t="n"/>
+      <c r="N20" s="23" t="n"/>
+      <c r="P20" s="29" t="n"/>
+      <c r="Q20" s="29" t="n"/>
       <c r="R20" s="29" t="n"/>
       <c r="S20" s="29" t="n"/>
       <c r="T20" s="29" t="n"/>
@@ -13587,4 +13944,796 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:W11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" style="41" min="1" max="1"/>
+    <col width="18" customWidth="1" style="41" min="2" max="2"/>
+    <col width="18" customWidth="1" style="41" min="3" max="3"/>
+    <col width="15.75" customWidth="1" style="41" min="4" max="4"/>
+    <col width="23.1299991607666" customWidth="1" style="41" min="5" max="5"/>
+    <col width="38" customWidth="1" style="41" min="6" max="6"/>
+    <col width="18" customWidth="1" style="41" min="7" max="7"/>
+    <col width="18" customWidth="1" style="41" min="8" max="8"/>
+    <col width="18" customWidth="1" style="41" min="9" max="9"/>
+    <col width="18" customWidth="1" style="41" min="10" max="10"/>
+    <col width="18" customWidth="1" style="41" min="11" max="11"/>
+    <col width="18" customWidth="1" style="41" min="12" max="12"/>
+    <col width="18" customWidth="1" style="41" min="13" max="13"/>
+    <col width="18" customWidth="1" style="41" min="14" max="14"/>
+    <col width="24" customWidth="1" style="41" min="15" max="15"/>
+    <col width="18" customWidth="1" style="41" min="16" max="16"/>
+    <col width="13" customWidth="1" style="41" min="17" max="17"/>
+    <col width="13" customWidth="1" style="41" min="18" max="18"/>
+    <col width="13" customWidth="1" style="41" min="19" max="19"/>
+    <col width="38" customWidth="1" style="41" min="20" max="20"/>
+    <col width="13" customWidth="1" style="41" min="21" max="21"/>
+    <col width="13" customWidth="1" style="41" min="22" max="22"/>
+    <col width="13" customWidth="1" style="41" min="23" max="23"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="28" t="inlineStr">
+        <is>
+          <t>First Name</t>
+        </is>
+      </c>
+      <c r="B1" s="28" t="inlineStr">
+        <is>
+          <t>Last Name</t>
+        </is>
+      </c>
+      <c r="C1" s="28" t="inlineStr">
+        <is>
+          <t>uid</t>
+        </is>
+      </c>
+      <c r="D1" s="28" t="inlineStr">
+        <is>
+          <t>Group Chat</t>
+        </is>
+      </c>
+      <c r="E1" s="28" t="inlineStr">
+        <is>
+          <t>Before Class Informing</t>
+        </is>
+      </c>
+      <c r="F1" s="28" t="inlineStr">
+        <is>
+          <t>Remark for Student</t>
+        </is>
+      </c>
+      <c r="G1" s="39" t="inlineStr">
+        <is>
+          <t>Parent Language</t>
+        </is>
+      </c>
+      <c r="H1" s="39" t="inlineStr">
+        <is>
+          <t>Class Attendance</t>
+        </is>
+      </c>
+      <c r="I1" s="39" t="inlineStr">
+        <is>
+          <t>Note-taking</t>
+        </is>
+      </c>
+      <c r="J1" s="39" t="inlineStr">
+        <is>
+          <t>Listening &amp; Focus</t>
+        </is>
+      </c>
+      <c r="K1" s="39" t="inlineStr">
+        <is>
+          <t>Participation</t>
+        </is>
+      </c>
+      <c r="L1" s="39" t="inlineStr">
+        <is>
+          <t>Practice Speed &amp; Accuracy</t>
+        </is>
+      </c>
+      <c r="M1" s="39" t="inlineStr">
+        <is>
+          <t>Proof Logic</t>
+        </is>
+      </c>
+      <c r="N1" s="39" t="inlineStr">
+        <is>
+          <t>Calculation</t>
+        </is>
+      </c>
+      <c r="O1" s="15" t="inlineStr">
+        <is>
+          <t>Additional Comment</t>
+        </is>
+      </c>
+      <c r="P1" s="39" t="inlineStr">
+        <is>
+          <t>Homework Reflection</t>
+        </is>
+      </c>
+      <c r="Q1" s="39" t="inlineStr">
+        <is>
+          <t>Send Status</t>
+        </is>
+      </c>
+      <c r="R1" s="28" t="inlineStr">
+        <is>
+          <t>Pre-quiz informing</t>
+        </is>
+      </c>
+      <c r="S1" s="28" t="inlineStr">
+        <is>
+          <t>Quiz Feedback</t>
+        </is>
+      </c>
+      <c r="T1" s="28" t="inlineStr">
+        <is>
+          <t>Second Feeback</t>
+        </is>
+      </c>
+      <c r="U1" s="28" t="inlineStr">
+        <is>
+          <t>Feedback</t>
+        </is>
+      </c>
+      <c r="V1" s="15" t="inlineStr">
+        <is>
+          <t>Send Error</t>
+        </is>
+      </c>
+      <c r="W1" s="15" t="inlineStr">
+        <is>
+          <t>Last Attempt</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>Andy</t>
+        </is>
+      </c>
+      <c r="B2" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Li</t>
+        </is>
+      </c>
+      <c r="C2" s="15" t="n">
+        <v>8125220</v>
+      </c>
+      <c r="D2" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="E2" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="F2" s="15" t="inlineStr">
+        <is>
+          <t>quiz 满分 5/8，孩子不太爱写过程，同时计算方面会有点不仔细，证明不太严谨，会漏步骤，需要先证明三角形全等，才可以用congruent part of congurent triangle are congruent</t>
+        </is>
+      </c>
+      <c r="G2" s="15" t="inlineStr">
+        <is>
+          <t>Chinese</t>
+        </is>
+      </c>
+      <c r="H2" s="15" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="I2" s="15" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J2" s="15" t="inlineStr">
+        <is>
+          <t>Focused</t>
+        </is>
+      </c>
+      <c r="K2" s="15" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="L2" s="15" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="U2" s="15" t="inlineStr">
+        <is>
+          <t>家长您好，我们目前已经完成了 Geometry Summer Camp 前半部分的课程内容。到目前为止，课程主要覆盖了平行线、三角形的基本性质、全等三角形、等腰三角形、角平分线、垂直平分线的性质，以及勾股定理等重要知识点。
+同时，学生们也完成了第一次 quiz。本次 quiz 满分为 8 分，包含 7 道选择题和 1 道证明题。证明题有 partial credit，如果证明题中错误较多，特别是错两处及以上，则可能无法获得该题分数。本次 quiz 的平均分为 6.9/8。整体来看，如果孩子的分数低于 6.5 分，建议您适当关注一下目前的学习掌握情况，尤其是计算细节和证明书写的规范性。
+接下来的 Geometry 学习会涉及更多计算，因此希望孩子们在做题时更加细心，注意步骤完整、计算准确。周四我们还会安排一次简单的小测验，一共 4 道题，主要检测学生对等腰三角形、角平分线、垂直平分线以及勾股定理的理解和运用。
+之后，我们将进入后半部分课程的学习，内容会包括三角函数、平行四边形、菱形、梯形、圆，以及相似三角形的证明。后半部分课程会有更多计算和综合应用，也会更加依赖前半部分知识的熟练掌握，因此希望同学们课后及时复习前面的重点内容，打好基础。
+本次 quiz 得分为 5/8，低于本次班级平均分 6.9/8，建议您最近多关注一下孩子对前半部分知识的掌握情况。从这次 quiz 和课堂情况来看，Andy 接下来可以重点关注做题时需要更主动地写出完整过程。计算细节也需要更加仔细。证明书写也需要更严谨，避免漏掉关键步骤。特别要注意先证明三角形全等，再使用对应边或对应角相等。结合课堂表现来看，Andy 笔记比较完整，听课比较专注，课堂参与度一般，练习完成情况不错。后续可以继续复习前半部分知识，并在计算准确性和证明步骤完整性上多检查。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="15" t="inlineStr">
+        <is>
+          <t>Athan</t>
+        </is>
+      </c>
+      <c r="B3" s="15" t="inlineStr">
+        <is>
+          <t>Tang</t>
+        </is>
+      </c>
+      <c r="C3" s="15" t="n">
+        <v>7877314</v>
+      </c>
+      <c r="D3" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="E3" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="F3" s="15" t="inlineStr">
+        <is>
+          <t>quiz 1满分 8/8，证明严谨，上课时常看apple watch或者出怪声会打扰到其余同学，希望家长可以督促一下</t>
+        </is>
+      </c>
+      <c r="G3" s="15" t="inlineStr">
+        <is>
+          <t>Chinese</t>
+        </is>
+      </c>
+      <c r="H3" s="15" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="I3" s="15" t="inlineStr">
+        <is>
+          <t>Okay</t>
+        </is>
+      </c>
+      <c r="J3" s="15" t="inlineStr">
+        <is>
+          <t>Sometimes Distracted</t>
+        </is>
+      </c>
+      <c r="K3" s="15" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="L3" s="15" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="U3" s="15" t="inlineStr">
+        <is>
+          <t>家长您好，我们目前已经完成了 Geometry Summer Camp 前半部分的课程内容。到目前为止，课程主要覆盖了平行线、三角形的基本性质、全等三角形、等腰三角形、角平分线、垂直平分线的性质，以及勾股定理等重要知识点。
+同时，学生们也完成了第一次 quiz。本次 quiz 满分为 8 分，包含 7 道选择题和 1 道证明题。证明题有 partial credit，如果证明题中错误较多，特别是错两处及以上，则可能无法获得该题分数。本次 quiz 的平均分为 6.9/8。整体来看，如果孩子的分数低于 6.5 分，建议您适当关注一下目前的学习掌握情况，尤其是计算细节和证明书写的规范性。
+接下来的 Geometry 学习会涉及更多计算，因此希望孩子们在做题时更加细心，注意步骤完整、计算准确。周四我们还会安排一次简单的小测验，一共 4 道题，主要检测学生对等腰三角形、角平分线、垂直平分线以及勾股定理的理解和运用。
+之后，我们将进入后半部分课程的学习，内容会包括三角函数、平行四边形、菱形、梯形、圆，以及相似三角形的证明。后半部分课程会有更多计算和综合应用，也会更加依赖前半部分知识的熟练掌握，因此希望同学们课后及时复习前面的重点内容，打好基础。
+本次 quiz 得分为 8/8，整体表现很不错，说明前半部分知识掌握比较扎实。Athan 这次表现比较扎实，后续可以继续保持，尤其是证明书写比较严谨。课堂专注和课堂习惯方面也需要您在家里配合提醒。可以继续保持目前严谨、完整的作答习惯。结合课堂表现来看，Athan 笔记还可以更加完整，有时会分心，课堂参与度一般，练习完成情况不错。后续可以继续复习前半部分知识，并在计算准确性和证明步骤完整性上多检查。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>Kangyou</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>Tong</t>
+        </is>
+      </c>
+      <c r="C4" s="15" t="n">
+        <v>8342525</v>
+      </c>
+      <c r="D4" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="E4" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="F4" s="15" t="inlineStr">
+        <is>
+          <t>quiz 5.5/8, 选择题错了两到，都是计算问题，不喜欢写过程，证明题在上课笔记的时候也不太喜欢写，同时证明题的reason需要明确用if, then的format去写，或者用课上说过的shortcut</t>
+        </is>
+      </c>
+      <c r="G4" s="15" t="inlineStr">
+        <is>
+          <t>Chinese</t>
+        </is>
+      </c>
+      <c r="H4" s="15" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="I4" s="15" t="inlineStr">
+        <is>
+          <t>Okay</t>
+        </is>
+      </c>
+      <c r="J4" s="15" t="inlineStr">
+        <is>
+          <t>Focused</t>
+        </is>
+      </c>
+      <c r="K4" s="15" t="inlineStr">
+        <is>
+          <t>Quiet</t>
+        </is>
+      </c>
+      <c r="L4" s="15" t="inlineStr">
+        <is>
+          <t>Okay</t>
+        </is>
+      </c>
+      <c r="U4" s="15" t="inlineStr">
+        <is>
+          <t>家长您好，我们目前已经完成了 Geometry Summer Camp 前半部分的课程内容。到目前为止，课程主要覆盖了平行线、三角形的基本性质、全等三角形、等腰三角形、角平分线、垂直平分线的性质，以及勾股定理等重要知识点。
+同时，学生们也完成了第一次 quiz。本次 quiz 满分为 8 分，包含 7 道选择题和 1 道证明题。证明题有 partial credit，如果证明题中错误较多，特别是错两处及以上，则可能无法获得该题分数。本次 quiz 的平均分为 6.9/8。整体来看，如果孩子的分数低于 6.5 分，建议您适当关注一下目前的学习掌握情况，尤其是计算细节和证明书写的规范性。
+接下来的 Geometry 学习会涉及更多计算，因此希望孩子们在做题时更加细心，注意步骤完整、计算准确。周四我们还会安排一次简单的小测验，一共 4 道题，主要检测学生对等腰三角形、角平分线、垂直平分线以及勾股定理的理解和运用。
+之后，我们将进入后半部分课程的学习，内容会包括三角函数、平行四边形、菱形、梯形、圆，以及相似三角形的证明。后半部分课程会有更多计算和综合应用，也会更加依赖前半部分知识的熟练掌握，因此希望同学们课后及时复习前面的重点内容，打好基础。
+本次 quiz 得分为 5.5/8，低于本次班级平均分 6.9/8，建议您最近多关注一下孩子对前半部分知识的掌握情况。从这次 quiz 和课堂情况来看，Kangyou 接下来可以重点关注做题时需要更主动地写出完整过程。计算细节也需要更加仔细。证明中的 reason 也需要写得更明确。结合课堂表现来看，Kangyou 笔记还可以更加完整，听课比较专注，课堂上比较安静，练习完成情况还可以继续提升。后续可以继续复习前半部分知识，并在计算准确性和证明步骤完整性上多检查。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>Ryan</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="inlineStr">
+        <is>
+          <t>Jiang</t>
+        </is>
+      </c>
+      <c r="C5" s="15" t="n">
+        <v>7881126</v>
+      </c>
+      <c r="D5" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="E5" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="G5" s="15" t="inlineStr">
+        <is>
+          <t>Chinese</t>
+        </is>
+      </c>
+      <c r="H5" s="15" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="I5" s="15" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J5" s="15" t="inlineStr">
+        <is>
+          <t>Focused</t>
+        </is>
+      </c>
+      <c r="K5" s="15" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="L5" s="15" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>Chengxuan</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>Song</t>
+        </is>
+      </c>
+      <c r="C6" s="15" t="n">
+        <v>8308069</v>
+      </c>
+      <c r="D6" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="E6" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="F6" s="15" t="inlineStr">
+        <is>
+          <t>quiz 7/8, 选择题全对，证明题有个错，需要明确是alternate interior angle are congruent， then two lines are parallel, 同时，学生在平行线对应的三种shape有些不牢固，需要孩子明确平行线该怎么对应哪几种special angle，不要被别的平行线干扰判断</t>
+        </is>
+      </c>
+      <c r="G6" s="15" t="inlineStr">
+        <is>
+          <t>Chinese</t>
+        </is>
+      </c>
+      <c r="H6" s="15" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="I6" s="15" t="inlineStr">
+        <is>
+          <t>Okay</t>
+        </is>
+      </c>
+      <c r="J6" s="15" t="inlineStr">
+        <is>
+          <t>Sometimes Distracted</t>
+        </is>
+      </c>
+      <c r="K6" s="15" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="L6" s="15" t="inlineStr">
+        <is>
+          <t>Okay</t>
+        </is>
+      </c>
+      <c r="U6" s="15" t="inlineStr">
+        <is>
+          <t>家长您好，我们目前已经完成了 Geometry Summer Camp 前半部分的课程内容。到目前为止，课程主要覆盖了平行线、三角形的基本性质、全等三角形、等腰三角形、角平分线、垂直平分线的性质，以及勾股定理等重要知识点。
+同时，学生们也完成了第一次 quiz。本次 quiz 满分为 8 分，包含 7 道选择题和 1 道证明题。证明题有 partial credit，如果证明题中错误较多，特别是错两处及以上，则可能无法获得该题分数。本次 quiz 的平均分为 6.9/8。整体来看，如果孩子的分数低于 6.5 分，建议您适当关注一下目前的学习掌握情况，尤其是计算细节和证明书写的规范性。
+接下来的 Geometry 学习会涉及更多计算，因此希望孩子们在做题时更加细心，注意步骤完整、计算准确。周四我们还会安排一次简单的小测验，一共 4 道题，主要检测学生对等腰三角形、角平分线、垂直平分线以及勾股定理的理解和运用。
+之后，我们将进入后半部分课程的学习，内容会包括三角函数、平行四边形、菱形、梯形、圆，以及相似三角形的证明。后半部分课程会有更多计算和综合应用，也会更加依赖前半部分知识的熟练掌握，因此希望同学们课后及时复习前面的重点内容，打好基础。
+本次 quiz 得分为 7/8，整体接近或达到本次班级平均水平。从这次 quiz 和课堂情况来看，Chengxuan 接下来可以重点关注选择题部分完成得很好。平行线相关证明中要清楚写出 alternate interior angles congruent 等关键理由。平行线对应的几种 special angle 图形也需要继续巩固，做题时不要被其他平行线干扰判断。结合课堂表现来看，Chengxuan 笔记还可以更加完整，有时会分心，课堂参与积极，练习完成情况还可以继续提升。后续可以继续复习前半部分知识，并在计算准确性和证明步骤完整性上多检查。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>Clarence</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+      <c r="C7" s="15" t="n">
+        <v>8389890</v>
+      </c>
+      <c r="D7" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="E7" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="F7" s="15" t="inlineStr">
+        <is>
+          <t>quiz 7/8, 选择题全对，证明题有个错，需要明确是alternate interior angle are congruent， then two lines are parallel, 同时，学生在平行线对应的三种shape有些不牢固，需要孩子明确平行线该怎么对应哪几种special angle，不要被别的平行线干扰判断</t>
+        </is>
+      </c>
+      <c r="G7" s="15" t="inlineStr">
+        <is>
+          <t>Chinese</t>
+        </is>
+      </c>
+      <c r="H7" s="15" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="I7" s="15" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J7" s="15" t="inlineStr">
+        <is>
+          <t>Focused</t>
+        </is>
+      </c>
+      <c r="K7" s="15" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="L7" s="15" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="U7" s="15" t="inlineStr">
+        <is>
+          <t>家长您好，我们目前已经完成了 Geometry Summer Camp 前半部分的课程内容。到目前为止，课程主要覆盖了平行线、三角形的基本性质、全等三角形、等腰三角形、角平分线、垂直平分线的性质，以及勾股定理等重要知识点。
+同时，学生们也完成了第一次 quiz。本次 quiz 满分为 8 分，包含 7 道选择题和 1 道证明题。证明题有 partial credit，如果证明题中错误较多，特别是错两处及以上，则可能无法获得该题分数。本次 quiz 的平均分为 6.9/8。整体来看，如果孩子的分数低于 6.5 分，建议您适当关注一下目前的学习掌握情况，尤其是计算细节和证明书写的规范性。
+接下来的 Geometry 学习会涉及更多计算，因此希望孩子们在做题时更加细心，注意步骤完整、计算准确。周四我们还会安排一次简单的小测验，一共 4 道题，主要检测学生对等腰三角形、角平分线、垂直平分线以及勾股定理的理解和运用。
+之后，我们将进入后半部分课程的学习，内容会包括三角函数、平行四边形、菱形、梯形、圆，以及相似三角形的证明。后半部分课程会有更多计算和综合应用，也会更加依赖前半部分知识的熟练掌握，因此希望同学们课后及时复习前面的重点内容，打好基础。
+本次 quiz 得分为 7/8，整体接近或达到本次班级平均水平。从这次 quiz 和课堂情况来看，Clarence 接下来可以重点关注选择题部分完成得很好。平行线相关证明中要清楚写出 alternate interior angles congruent 等关键理由。平行线对应的几种 special angle 图形也需要继续巩固，做题时不要被其他平行线干扰判断。结合课堂表现来看，Clarence 笔记比较完整，听课比较专注，课堂参与积极，练习完成情况不错。后续可以继续复习前半部分知识，并在计算准确性和证明步骤完整性上多检查。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="15" t="inlineStr">
+        <is>
+          <t>Annika</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="inlineStr">
+        <is>
+          <t>Srivastava</t>
+        </is>
+      </c>
+      <c r="C8" s="15" t="n">
+        <v>8392845</v>
+      </c>
+      <c r="D8" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="E8" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="F8" s="15" t="inlineStr">
+        <is>
+          <t>Perfect in quiz 1, recieve 8/8, proof is rigrous and also concise</t>
+        </is>
+      </c>
+      <c r="G8" s="15" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="H8" s="15" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="I8" s="15" t="inlineStr">
+        <is>
+          <t>Excellent</t>
+        </is>
+      </c>
+      <c r="J8" s="15" t="inlineStr">
+        <is>
+          <t>Very Focused</t>
+        </is>
+      </c>
+      <c r="K8" s="15" t="inlineStr">
+        <is>
+          <t>Very Active</t>
+        </is>
+      </c>
+      <c r="L8" s="15" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="U8" s="15" t="inlineStr">
+        <is>
+          <t>Hello parents, we have now completed the first half of our Geometry Summer Camp. So far, the course has covered parallel lines, basic triangle properties, congruent triangles, isosceles triangles, angle bisectors, perpendicular bisectors, and the Pythagorean Theorem.
+Students have also completed their first quiz. The quiz was out of 8 points and included 7 multiple-choice questions and 1 proof question. The proof question allowed partial credit, but students could lose the full proof score if there were two or more significant mistakes. The class average was 6.9/8. In general, if a student scored below 6.5, it may be helpful to pay closer attention to their current understanding, especially their calculation accuracy and proof-writing structure.
+As we move forward, Geometry will involve more calculation, so students will need to be more careful with their work, show complete steps, and check their answers closely. On Thursday, we will also have a short quiz with 4 questions. This quiz will check students' understanding and application of isosceles triangles, angle bisectors, perpendicular bisectors, and the Pythagorean Theorem.
+After that, we will begin the second half of the course, which will include trigonometry, parallelograms, rhombi, trapezoids, circles, and proofs involving similar triangles. The second half of the course will include more calculations and more mixed applications, so students will need to be comfortable with the topics from the first half. I encourage students to review these key concepts regularly so they can build a strong foundation for the remaining lessons.
+The quiz score was 8/8, which is a strong result and shows solid understanding of the first-half topics. Annika can build from this by continuing to focus on maintaining the strong quiz performance, and keeping proof writing rigorous and concise. During class, Annika took excellent notes, stayed very focused, participated very actively, and showed strong accuracy on practice problems. Going forward, reviewing the first-half topics while checking calculation details and proof structure carefully will help keep the foundation strong.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>Beichen</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="inlineStr">
+        <is>
+          <t>Xin</t>
+        </is>
+      </c>
+      <c r="C9" s="15" t="n">
+        <v>7904958</v>
+      </c>
+      <c r="D9" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="E9" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="F9" s="15" t="inlineStr">
+        <is>
+          <t>quiz 1, 8/8, 证明严谨，也都也写了过程</t>
+        </is>
+      </c>
+      <c r="G9" s="15" t="inlineStr">
+        <is>
+          <t>Chinese</t>
+        </is>
+      </c>
+      <c r="H9" s="15" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="I9" s="15" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J9" s="15" t="inlineStr">
+        <is>
+          <t>Focused</t>
+        </is>
+      </c>
+      <c r="K9" s="15" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="L9" s="15" t="inlineStr">
+        <is>
+          <t>Okay</t>
+        </is>
+      </c>
+      <c r="U9" s="15" t="inlineStr">
+        <is>
+          <t>家长您好，我们目前已经完成了 Geometry Summer Camp 前半部分的课程内容。到目前为止，课程主要覆盖了平行线、三角形的基本性质、全等三角形、等腰三角形、角平分线、垂直平分线的性质，以及勾股定理等重要知识点。
+同时，学生们也完成了第一次 quiz。本次 quiz 满分为 8 分，包含 7 道选择题和 1 道证明题。证明题有 partial credit，如果证明题中错误较多，特别是错两处及以上，则可能无法获得该题分数。本次 quiz 的平均分为 6.9/8。整体来看，如果孩子的分数低于 6.5 分，建议您适当关注一下目前的学习掌握情况，尤其是计算细节和证明书写的规范性。
+接下来的 Geometry 学习会涉及更多计算，因此希望孩子们在做题时更加细心，注意步骤完整、计算准确。周四我们还会安排一次简单的小测验，一共 4 道题，主要检测学生对等腰三角形、角平分线、垂直平分线以及勾股定理的理解和运用。
+之后，我们将进入后半部分课程的学习，内容会包括三角函数、平行四边形、菱形、梯形、圆，以及相似三角形的证明。后半部分课程会有更多计算和综合应用，也会更加依赖前半部分知识的熟练掌握，因此希望同学们课后及时复习前面的重点内容，打好基础。
+本次 quiz 得分为 8/8，整体表现很不错，说明前半部分知识掌握比较扎实。Beichen 这次表现比较扎实，后续可以继续保持，尤其是证明书写比较严谨。可以继续保持目前严谨、完整的作答习惯。结合课堂表现来看，Beichen 笔记比较完整，听课比较专注，课堂参与度一般，练习完成情况还可以继续提升。后续可以继续复习前半部分知识，并在计算准确性和证明步骤完整性上多检查。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="15" t="inlineStr">
+        <is>
+          <t>Aaron</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>Cheng</t>
+        </is>
+      </c>
+      <c r="C10" s="15" t="n">
+        <v>8347973</v>
+      </c>
+      <c r="D10" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="E10" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="F10" s="15" t="inlineStr">
+        <is>
+          <t>quiz 1， 7.5/8, 选择题全对，证明题在reason方面有点小欠缺，需要清晰写出因为平行，所以alternative interior angle are congruent</t>
+        </is>
+      </c>
+      <c r="G10" s="15" t="inlineStr">
+        <is>
+          <t>Chinese</t>
+        </is>
+      </c>
+      <c r="H10" s="15" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="I10" s="15" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J10" s="15" t="inlineStr">
+        <is>
+          <t>Focused</t>
+        </is>
+      </c>
+      <c r="K10" s="15" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="L10" s="15" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="U10" s="15" t="inlineStr">
+        <is>
+          <t>家长您好，我们目前已经完成了 Geometry Summer Camp 前半部分的课程内容。到目前为止，课程主要覆盖了平行线、三角形的基本性质、全等三角形、等腰三角形、角平分线、垂直平分线的性质，以及勾股定理等重要知识点。
+同时，学生们也完成了第一次 quiz。本次 quiz 满分为 8 分，包含 7 道选择题和 1 道证明题。证明题有 partial credit，如果证明题中错误较多，特别是错两处及以上，则可能无法获得该题分数。本次 quiz 的平均分为 6.9/8。整体来看，如果孩子的分数低于 6.5 分，建议您适当关注一下目前的学习掌握情况，尤其是计算细节和证明书写的规范性。
+接下来的 Geometry 学习会涉及更多计算，因此希望孩子们在做题时更加细心，注意步骤完整、计算准确。周四我们还会安排一次简单的小测验，一共 4 道题，主要检测学生对等腰三角形、角平分线、垂直平分线以及勾股定理的理解和运用。
+之后，我们将进入后半部分课程的学习，内容会包括三角函数、平行四边形、菱形、梯形、圆，以及相似三角形的证明。后半部分课程会有更多计算和综合应用，也会更加依赖前半部分知识的熟练掌握，因此希望同学们课后及时复习前面的重点内容，打好基础。
+本次 quiz 得分为 7.5/8，整体表现很不错，说明前半部分知识掌握比较扎实。Aaron 这次表现比较扎实，后续可以继续保持，尤其是选择题部分完成得很好。证明中的 reason 也需要写得更明确。结合课堂表现来看，Aaron 笔记比较完整，听课比较专注，课堂参与积极，练习完成情况不错。后续可以继续复习前半部分知识，并在计算准确性和证明步骤完整性上多检查。</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>Luke</t>
+        </is>
+      </c>
+      <c r="B11" s="15" t="inlineStr">
+        <is>
+          <t>Li</t>
+        </is>
+      </c>
+      <c r="C11" s="15" t="n">
+        <v>8194394</v>
+      </c>
+      <c r="D11" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="E11" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="F11" s="15" t="inlineStr">
+        <is>
+          <t>quiz 7/8, 选择题全对，证明题有个错，需要明确是alternate interior angle are congruent， then two lines are parallel, 同时，学生在平行线对应的三种shape有些不牢固，需要孩子明确平行线该怎么对应哪几种special angle，不要被别的平行线干扰判断</t>
+        </is>
+      </c>
+      <c r="G11" s="15" t="inlineStr">
+        <is>
+          <t>Chinese</t>
+        </is>
+      </c>
+      <c r="H11" s="15" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="I11" s="15" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J11" s="15" t="inlineStr">
+        <is>
+          <t>Focused</t>
+        </is>
+      </c>
+      <c r="K11" s="15" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="L11" s="15" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="U11" s="15" t="inlineStr">
+        <is>
+          <t>家长您好，我们目前已经完成了 Geometry Summer Camp 前半部分的课程内容。到目前为止，课程主要覆盖了平行线、三角形的基本性质、全等三角形、等腰三角形、角平分线、垂直平分线的性质，以及勾股定理等重要知识点。
+同时，学生们也完成了第一次 quiz。本次 quiz 满分为 8 分，包含 7 道选择题和 1 道证明题。证明题有 partial credit，如果证明题中错误较多，特别是错两处及以上，则可能无法获得该题分数。本次 quiz 的平均分为 6.9/8。整体来看，如果孩子的分数低于 6.5 分，建议您适当关注一下目前的学习掌握情况，尤其是计算细节和证明书写的规范性。
+接下来的 Geometry 学习会涉及更多计算，因此希望孩子们在做题时更加细心，注意步骤完整、计算准确。周四我们还会安排一次简单的小测验，一共 4 道题，主要检测学生对等腰三角形、角平分线、垂直平分线以及勾股定理的理解和运用。
+之后，我们将进入后半部分课程的学习，内容会包括三角函数、平行四边形、菱形、梯形、圆，以及相似三角形的证明。后半部分课程会有更多计算和综合应用，也会更加依赖前半部分知识的熟练掌握，因此希望同学们课后及时复习前面的重点内容，打好基础。
+本次 quiz 得分为 7/8，整体接近或达到本次班级平均水平。从这次 quiz 和课堂情况来看，Luke 接下来可以重点关注选择题部分完成得很好。平行线相关证明中要清楚写出 alternate interior angles congruent 等关键理由。平行线对应的几种 special angle 图形也需要继续巩固，做题时不要被其他平行线干扰判断。结合课堂表现来看，Luke 笔记比较完整，听课比较专注，课堂参与积极，练习完成情况不错。后续可以继续复习前半部分知识，并在计算准确性和证明步骤完整性上多检查。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add local frontend docs and CLI row selection
</commit_message>
<xml_diff>
--- a/Geo_TTh_Student_Script_fixed_rows_only.xlsx
+++ b/Geo_TTh_Student_Script_fixed_rows_only.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowHeight="12255" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Geo WF" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="AMC10 Intro" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Geo TTh" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Geo MTWThF" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Geo WF" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AMC10 Intro" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Geo TTh" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Geo MTWThF" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Geo WF'!$A$1:$AD$52</definedName>
@@ -1159,7 +1159,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE52"/>
+  <dimension ref="A1:AE55"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6285714285714" defaultRowHeight="12.75"/>
   <cols>
     <col width="18" customWidth="1" style="1" min="1" max="1"/>
@@ -1348,8 +1348,10 @@
           <t>Zhang</t>
         </is>
       </c>
-      <c r="C2" s="0" t="n">
-        <v>8288137</v>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>8288137</t>
+        </is>
       </c>
       <c r="D2" s="0" t="b">
         <v>0</v>
@@ -1394,7 +1396,13 @@
       </c>
       <c r="Q2" s="0" t="n"/>
       <c r="T2" s="0" t="n"/>
-      <c r="U2" s="0" t="n"/>
+      <c r="U2" s="0" t="inlineStr">
+        <is>
+          <t>今天课堂主要围绕本节几何课的核心概念、例题讲解和课堂练习展开。
+从课堂补充记录来看，Wenjie 在课堂记录和做题习惯整体比较稳定。
+如果您还有任何问题，可以直接在群里问我，我会尽快回复。</t>
+        </is>
+      </c>
       <c r="V2" s="0" t="n"/>
       <c r="W2" s="0" t="n"/>
       <c r="X2" s="5" t="n"/>
@@ -1414,8 +1422,10 @@
           <t>Wang</t>
         </is>
       </c>
-      <c r="C3" s="0" t="n">
-        <v>7878730</v>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>7878730</t>
+        </is>
       </c>
       <c r="D3" s="0" t="b">
         <v>1</v>
@@ -1460,7 +1470,13 @@
       </c>
       <c r="Q3" s="0" t="n"/>
       <c r="T3" s="0" t="n"/>
-      <c r="U3" s="0" t="n"/>
+      <c r="U3" s="0" t="inlineStr">
+        <is>
+          <t>今天课堂主要围绕本节几何课的核心概念、例题讲解和课堂练习展开。
+从课堂补充记录来看，Catherine 在课堂记录和做题习惯整体比较稳定。
+如果您还有任何问题，可以直接在群里问我，我会尽快回复。</t>
+        </is>
+      </c>
       <c r="V3" s="0" t="n"/>
       <c r="W3" s="0" t="n"/>
       <c r="X3" s="5" t="n"/>
@@ -1480,8 +1496,10 @@
           <t>Lin</t>
         </is>
       </c>
-      <c r="C4" s="0" t="n">
-        <v>7879477</v>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>7879477</t>
+        </is>
       </c>
       <c r="D4" s="0" t="b">
         <v>1</v>
@@ -1526,7 +1544,13 @@
       </c>
       <c r="Q4" s="0" t="n"/>
       <c r="T4" s="0" t="n"/>
-      <c r="U4" s="0" t="n"/>
+      <c r="U4" s="0" t="inlineStr">
+        <is>
+          <t>今天课堂主要围绕本节几何课的核心概念、例题讲解和课堂练习展开。
+从课堂补充记录来看，Maxwell 在证明书写方面有不错的基础，课堂记录和做题习惯整体比较稳定。
+如果您还有任何问题，可以直接在群里问我，我会尽快回复。</t>
+        </is>
+      </c>
       <c r="V4" s="0" t="n"/>
       <c r="W4" s="0" t="n"/>
       <c r="X4" s="5" t="n"/>
@@ -1546,8 +1570,10 @@
           <t>Sanjay</t>
         </is>
       </c>
-      <c r="C5" s="0" t="n">
-        <v>7899198</v>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>7899198</t>
+        </is>
       </c>
       <c r="D5" s="0" t="b">
         <v>1</v>
@@ -1591,6 +1617,13 @@
         </is>
       </c>
       <c r="Q5" s="0" t="n"/>
+      <c r="U5" s="0" t="inlineStr">
+        <is>
+          <t>In today's class, we reviewed the main geometry ideas for the lesson, worked through examples, and practiced applying the methods in class.
+Nikhil had a steady class today and took good notes, stayed focused, participated at an average level, and did well on practice problems. Continuing to build proof logic while checking details carefully will be helpful.
+If you have any questions, feel free to ask me directly in the group chat. I will reply as soon as possible.</t>
+        </is>
+      </c>
       <c r="V5" s="0" t="n"/>
       <c r="W5" s="0" t="n"/>
       <c r="X5" s="6" t="n"/>
@@ -1610,8 +1643,10 @@
           <t>Wang</t>
         </is>
       </c>
-      <c r="C6" s="0" t="n">
-        <v>8397412</v>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>8397412</t>
+        </is>
       </c>
       <c r="D6" s="0" t="b">
         <v>1</v>
@@ -1656,7 +1691,13 @@
       </c>
       <c r="Q6" s="0" t="n"/>
       <c r="T6" s="0" t="n"/>
-      <c r="U6" s="0" t="n"/>
+      <c r="U6" s="0" t="inlineStr">
+        <is>
+          <t>今天课堂主要围绕本节几何课的核心概念、例题讲解和课堂练习展开。
+从课堂补充记录来看，Audrey 在课堂记录和做题习惯整体比较稳定。
+如果您还有任何问题，可以直接在群里问我，我会尽快回复。</t>
+        </is>
+      </c>
       <c r="V6" s="0" t="n"/>
       <c r="W6" s="0" t="n"/>
       <c r="X6" s="5" t="n"/>
@@ -1676,8 +1717,10 @@
           <t>Wang</t>
         </is>
       </c>
-      <c r="C7" s="0" t="n">
-        <v>8395094</v>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>8395094</t>
+        </is>
       </c>
       <c r="D7" s="0" t="b">
         <v>1</v>
@@ -1722,7 +1765,13 @@
       </c>
       <c r="Q7" s="0" t="n"/>
       <c r="T7" s="0" t="n"/>
-      <c r="U7" s="0" t="n"/>
+      <c r="U7" s="0" t="inlineStr">
+        <is>
+          <t>今天课堂主要围绕本节几何课的核心概念、例题讲解和课堂练习展开。
+从课堂补充记录来看，Ruoxi 在课堂记录和做题习惯整体比较稳定。
+如果您还有任何问题，可以直接在群里问我，我会尽快回复。</t>
+        </is>
+      </c>
       <c r="V7" s="0" t="n"/>
       <c r="W7" s="0" t="n"/>
       <c r="X7" s="5" t="n"/>
@@ -1742,8 +1791,10 @@
           <t>Zhang</t>
         </is>
       </c>
-      <c r="C8" s="0" t="n">
-        <v>8266668</v>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>8266668</t>
+        </is>
       </c>
       <c r="D8" s="0" t="b">
         <v>0</v>
@@ -1788,7 +1839,13 @@
       </c>
       <c r="Q8" s="0" t="n"/>
       <c r="T8" s="0" t="n"/>
-      <c r="U8" s="0" t="n"/>
+      <c r="U8" s="0" t="inlineStr">
+        <is>
+          <t>今天课堂主要围绕本节几何课的核心概念、例题讲解和课堂练习展开。
+从课堂补充记录来看，Mattias 在课堂专注和课堂习惯方面还可以继续调整，课堂记录和做题过程还可以更加完整。
+如果您还有任何问题，可以直接在群里问我，我会尽快回复。</t>
+        </is>
+      </c>
       <c r="V8" s="0" t="n"/>
       <c r="W8" s="0" t="n"/>
       <c r="X8" s="6" t="n"/>
@@ -1808,8 +1865,10 @@
           <t>Soldner</t>
         </is>
       </c>
-      <c r="C9" s="0" t="n">
-        <v>7938774</v>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>7938774</t>
+        </is>
       </c>
       <c r="D9" s="0" t="b">
         <v>0</v>
@@ -1853,7 +1912,13 @@
         </is>
       </c>
       <c r="Q9" s="0" t="n"/>
-      <c r="U9" s="0" t="n"/>
+      <c r="U9" s="0" t="inlineStr">
+        <is>
+          <t>In today's class, we reviewed the main geometry ideas for the lesson, worked through examples, and practiced applying the methods in class.
+Adelynn had a steady class today and took good notes, stayed focused, participated at an average level, and did well on practice problems. Continuing to build proof logic while checking details carefully will be helpful.
+If you have any questions, feel free to ask me directly in the group chat. I will reply as soon as possible.</t>
+        </is>
+      </c>
       <c r="V9" s="0" t="n"/>
       <c r="W9" s="0" t="n"/>
       <c r="X9" s="5" t="n"/>
@@ -1862,7 +1927,7 @@
       <c r="AD9" s="7" t="n"/>
       <c r="AE9" s="0" t="n"/>
     </row>
-    <row r="10">
+    <row r="10" s="1">
       <c r="A10" s="0" t="inlineStr">
         <is>
           <t>Sophia</t>
@@ -1873,11 +1938,21 @@
           <t>Sun</t>
         </is>
       </c>
-      <c r="C10" s="0" t="n"/>
-      <c r="D10" s="0" t="n"/>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>8162357</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="b">
+        <v>1</v>
+      </c>
       <c r="E10" s="0" t="n"/>
       <c r="F10" s="0" t="n"/>
-      <c r="G10" s="0" t="n"/>
+      <c r="G10" s="0" t="inlineStr">
+        <is>
+          <t>Chinese</t>
+        </is>
+      </c>
       <c r="H10" s="0" t="n"/>
       <c r="I10" s="0" t="n"/>
       <c r="J10" s="0" t="n"/>
@@ -1890,7 +1965,13 @@
         </is>
       </c>
       <c r="T10" s="0" t="n"/>
-      <c r="U10" s="0" t="n"/>
+      <c r="U10" s="0" t="inlineStr">
+        <is>
+          <t>In today's class, we reviewed the main geometry ideas for the lesson, worked through examples, and practiced applying the methods in class.
+Sophia's classroom notes have been recorded for today's lesson.
+If you have any questions, feel free to ask me directly in the group chat. I will reply as soon as possible.</t>
+        </is>
+      </c>
       <c r="V10" s="0" t="n"/>
       <c r="W10" s="0" t="n"/>
       <c r="X10" s="5" t="n"/>
@@ -2913,6 +2994,144 @@
       <c r="AC52" s="6" t="n"/>
       <c r="AD52" s="6" t="n"/>
       <c r="AE52" s="0" t="n"/>
+    </row>
+    <row r="53" s="1">
+      <c r="A53" s="0" t="inlineStr">
+        <is>
+          <t>Steven</t>
+        </is>
+      </c>
+      <c r="B53" s="0" t="inlineStr">
+        <is>
+          <t>Xu</t>
+        </is>
+      </c>
+      <c r="C53" s="0" t="inlineStr">
+        <is>
+          <t>8226195</t>
+        </is>
+      </c>
+      <c r="D53" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="E53" s="0" t="n"/>
+      <c r="F53" s="0" t="n"/>
+      <c r="G53" s="0" t="inlineStr">
+        <is>
+          <t>Chinese</t>
+        </is>
+      </c>
+      <c r="H53" s="0" t="n"/>
+      <c r="I53" s="0" t="n"/>
+      <c r="J53" s="0" t="n"/>
+      <c r="K53" s="0" t="n"/>
+      <c r="L53" s="0" t="n"/>
+      <c r="Q53" s="0" t="n"/>
+      <c r="S53" s="0" t="n"/>
+      <c r="T53" s="0" t="n"/>
+      <c r="U53" s="0" t="n"/>
+      <c r="V53" s="0" t="n"/>
+      <c r="W53" s="0" t="n"/>
+      <c r="X53" s="5" t="n"/>
+      <c r="Y53" s="0" t="n"/>
+      <c r="Z53" s="0" t="n"/>
+      <c r="AA53" s="0" t="n"/>
+      <c r="AB53" s="6" t="n"/>
+      <c r="AC53" s="6" t="n"/>
+      <c r="AD53" s="6" t="n"/>
+      <c r="AE53" s="0" t="n"/>
+    </row>
+    <row r="54" s="1">
+      <c r="A54" s="0" t="inlineStr">
+        <is>
+          <t>Judy</t>
+        </is>
+      </c>
+      <c r="B54" s="0" t="inlineStr">
+        <is>
+          <t>Cai</t>
+        </is>
+      </c>
+      <c r="C54" s="0" t="inlineStr">
+        <is>
+          <t>7990237</t>
+        </is>
+      </c>
+      <c r="D54" s="0" t="b">
+        <v>0</v>
+      </c>
+      <c r="E54" s="0" t="n"/>
+      <c r="F54" s="0" t="n"/>
+      <c r="G54" s="0" t="inlineStr">
+        <is>
+          <t>Chinese</t>
+        </is>
+      </c>
+      <c r="H54" s="0" t="n"/>
+      <c r="I54" s="0" t="n"/>
+      <c r="J54" s="0" t="n"/>
+      <c r="K54" s="0" t="n"/>
+      <c r="L54" s="0" t="n"/>
+      <c r="Q54" s="0" t="n"/>
+      <c r="S54" s="0" t="n"/>
+      <c r="T54" s="0" t="n"/>
+      <c r="U54" s="0" t="n"/>
+      <c r="V54" s="0" t="n"/>
+      <c r="W54" s="0" t="n"/>
+      <c r="X54" s="5" t="n"/>
+      <c r="Y54" s="0" t="n"/>
+      <c r="Z54" s="0" t="n"/>
+      <c r="AA54" s="0" t="n"/>
+      <c r="AB54" s="6" t="n"/>
+      <c r="AC54" s="6" t="n"/>
+      <c r="AD54" s="6" t="n"/>
+      <c r="AE54" s="0" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="0" t="inlineStr">
+        <is>
+          <t>Daisy</t>
+        </is>
+      </c>
+      <c r="B55" s="0" t="inlineStr">
+        <is>
+          <t>Chen</t>
+        </is>
+      </c>
+      <c r="C55" s="0" t="inlineStr">
+        <is>
+          <t>8020458</t>
+        </is>
+      </c>
+      <c r="D55" s="0" t="b">
+        <v>0</v>
+      </c>
+      <c r="E55" s="0" t="n"/>
+      <c r="F55" s="0" t="n"/>
+      <c r="G55" s="0" t="inlineStr">
+        <is>
+          <t>Chinese</t>
+        </is>
+      </c>
+      <c r="H55" s="0" t="n"/>
+      <c r="I55" s="0" t="n"/>
+      <c r="J55" s="0" t="n"/>
+      <c r="K55" s="0" t="n"/>
+      <c r="L55" s="0" t="n"/>
+      <c r="Q55" s="0" t="n"/>
+      <c r="S55" s="0" t="n"/>
+      <c r="T55" s="0" t="n"/>
+      <c r="U55" s="0" t="n"/>
+      <c r="V55" s="0" t="n"/>
+      <c r="W55" s="0" t="n"/>
+      <c r="X55" s="5" t="n"/>
+      <c r="Y55" s="0" t="n"/>
+      <c r="Z55" s="0" t="n"/>
+      <c r="AA55" s="0" t="n"/>
+      <c r="AB55" s="6" t="n"/>
+      <c r="AC55" s="6" t="n"/>
+      <c r="AD55" s="6" t="n"/>
+      <c r="AE55" s="0" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:AD52"/>
@@ -10225,7 +10444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE11"/>
+  <dimension ref="A1:AE12"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="12.75"/>
   <cols>
     <col width="18" customWidth="1" style="1" min="1" max="1"/>
@@ -10414,8 +10633,10 @@
           <t xml:space="preserve"> Li</t>
         </is>
       </c>
-      <c r="C2" s="0" t="n">
-        <v>8125220</v>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>8125220</t>
+        </is>
       </c>
       <c r="D2" s="0" t="b">
         <v>0</v>
@@ -10538,8 +10759,10 @@
           <t>Tang</t>
         </is>
       </c>
-      <c r="C3" s="0" t="n">
-        <v>7877314</v>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>7877314</t>
+        </is>
       </c>
       <c r="D3" s="0" t="b">
         <v>1</v>
@@ -10662,8 +10885,10 @@
           <t>Tong</t>
         </is>
       </c>
-      <c r="C4" s="0" t="n">
-        <v>8342525</v>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>8342525</t>
+        </is>
       </c>
       <c r="D4" s="0" t="b">
         <v>1</v>
@@ -10786,8 +11011,10 @@
           <t>Jiang</t>
         </is>
       </c>
-      <c r="C5" s="0" t="n">
-        <v>7881126</v>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>7881126</t>
+        </is>
       </c>
       <c r="D5" s="0" t="b">
         <v>0</v>
@@ -10836,7 +11063,7 @@
           <t>2026-06-19T01:34:26</t>
         </is>
       </c>
-      <c r="X5" s="6" t="inlineStr"/>
+      <c r="X5" s="6" t="n"/>
       <c r="AB5" s="6" t="inlineStr">
         <is>
           <t>家长您好，我们目前已经完成了 Geometry Summer Camp 前半部分的课程内容。到目前为止，课程主要覆盖了平行线、三角形的基本性质、全等三角形、等腰三角形、角平分线、垂直平分线的性质，以及勾股定理等重要知识点。
@@ -10875,8 +11102,10 @@
           <t>Song</t>
         </is>
       </c>
-      <c r="C6" s="0" t="n">
-        <v>8308069</v>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>8308069</t>
+        </is>
       </c>
       <c r="D6" s="0" t="b">
         <v>1</v>
@@ -10999,8 +11228,10 @@
           <t>Tan</t>
         </is>
       </c>
-      <c r="C7" s="0" t="n">
-        <v>8389890</v>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>8389890</t>
+        </is>
       </c>
       <c r="D7" s="0" t="b">
         <v>1</v>
@@ -11123,8 +11354,10 @@
           <t>Srivastava</t>
         </is>
       </c>
-      <c r="C8" s="0" t="n">
-        <v>8392845</v>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>8392845</t>
+        </is>
       </c>
       <c r="D8" s="0" t="b">
         <v>1</v>
@@ -11247,8 +11480,10 @@
           <t>Xin</t>
         </is>
       </c>
-      <c r="C9" s="0" t="n">
-        <v>7904958</v>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>7904958</t>
+        </is>
       </c>
       <c r="D9" s="0" t="b">
         <v>0</v>
@@ -11366,8 +11601,10 @@
           <t>Cheng</t>
         </is>
       </c>
-      <c r="C10" s="0" t="n">
-        <v>8347973</v>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>8347973</t>
+        </is>
       </c>
       <c r="D10" s="0" t="b">
         <v>1</v>
@@ -11490,8 +11727,10 @@
           <t>Li</t>
         </is>
       </c>
-      <c r="C11" s="0" t="n">
-        <v>8194394</v>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>8194394</t>
+        </is>
       </c>
       <c r="D11" s="0" t="b">
         <v>0</v>
@@ -11576,14 +11815,38 @@
 如果您还有任何问题，可以直接在群里问我，我会尽快回复。</t>
         </is>
       </c>
-      <c r="AB11" s="6" t="inlineStr"/>
-      <c r="AC11" s="6" t="inlineStr"/>
+      <c r="AB11" s="6" t="n"/>
+      <c r="AC11" s="6" t="n"/>
       <c r="AD11" s="6" t="n"/>
       <c r="AE11" s="0" t="inlineStr">
         <is>
           <t>6.4/9</t>
         </is>
       </c>
+    </row>
+    <row r="12" ht="409.5" customHeight="1" s="1">
+      <c r="A12" s="0" t="n"/>
+      <c r="B12" s="0" t="n"/>
+      <c r="C12" s="0" t="n"/>
+      <c r="D12" s="0" t="n"/>
+      <c r="E12" s="0" t="n"/>
+      <c r="F12" s="0" t="n"/>
+      <c r="G12" s="0" t="n"/>
+      <c r="H12" s="0" t="n"/>
+      <c r="I12" s="0" t="n"/>
+      <c r="J12" s="0" t="n"/>
+      <c r="K12" s="0" t="n"/>
+      <c r="L12" s="0" t="n"/>
+      <c r="Q12" s="0" t="n"/>
+      <c r="T12" s="0" t="n"/>
+      <c r="U12" s="0" t="n"/>
+      <c r="V12" s="0" t="n"/>
+      <c r="W12" s="0" t="n"/>
+      <c r="X12" s="5" t="n"/>
+      <c r="AB12" s="6" t="n"/>
+      <c r="AC12" s="6" t="n"/>
+      <c r="AD12" s="6" t="n"/>
+      <c r="AE12" s="0" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>